<commit_message>
Batch 5 reviewed and applied: out/esES.txt updated
382 lines approved as proposed, 9 with Bleu's Spanish. Catalyst Field is
now campo catalizador and Regen Field campo de regeneración; bola cebo,
paso de sombra, mejora (trait) and reequipar added to the glossary.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work/batch5/batch5-review.xlsx
+++ b/work/batch5/batch5-review.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maost\AppData\Local\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\[01] Martin\[07] Claude Code\NS2-Spanish-Translation\work\batch5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A044B155-17B1-4254-8F99-228004B0C28F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{640AEC7D-AA94-47DD-BDA6-4567A569E7C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6DD209BF-CDF2-4E8A-A1E5-09B7D78720A2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{6DD209BF-CDF2-4E8A-A1E5-09B7D78720A2}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2491" uniqueCount="1462">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2896" uniqueCount="1477">
   <si>
     <t>Section</t>
   </si>
@@ -4434,6 +4434,51 @@
   </si>
   <si>
     <t>Flagged left</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Use my Spanish</t>
+  </si>
+  <si>
+    <t>Hace que el Fade pase parcialmente a otra dimensión y vuele por el aire a muy alta velocidad. ¡Requiere mucha energía!</t>
+  </si>
+  <si>
+    <t>The joke on blinking is lost. Other spanish translations that have abilities called blink don't literally translate it since it sounds bad in spanish.</t>
+  </si>
+  <si>
+    <t>CAMPO CATALIZADOR</t>
+  </si>
+  <si>
+    <t>We've translated catalyst pack literally too, so this follows.</t>
+  </si>
+  <si>
+    <t>Aplasta a un enemigo con la culata del rifle. (Aquí va un chiste con la palabra 'culo')</t>
+  </si>
+  <si>
+    <t>Corrected the joke to work in spanish. Slightly more risqué because 'culo' is akin to 'ass' but definitely pg13.</t>
+  </si>
+  <si>
+    <t>Vuela a cualquier alien lo bastante tonto como para ponerse a distancia de ser acariciado.</t>
+  </si>
+  <si>
+    <t>Adjusted wording</t>
+  </si>
+  <si>
+    <t>Desbloquea las habilidades de apoyo del Exotraje: campo de nano-escudo, campo catalizador y campo de regeneración.</t>
+  </si>
+  <si>
+    <t>Emite un impulso catalizador sobre cada Marine a menos de 8 metros que no haya sido potenciado en los últimos 4 segundos. Solo Marines; no afecta a los Exotrajes. El efecto dura 5 segundos. Enfriamiento de 90 segundos.</t>
+  </si>
+  <si>
+    <t>Campo catalizador.</t>
+  </si>
+  <si>
+    <t>Campo de regeneración</t>
+  </si>
+  <si>
+    <t>Marcar Mapa</t>
   </si>
 </sst>
 </file>
@@ -4994,7 +5039,7 @@
       </c>
       <c r="B10" s="14">
         <f>COUNTA(Review!J2:J392)</f>
-        <v>0</v>
+        <v>391</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -5003,7 +5048,7 @@
       </c>
       <c r="B11" s="14">
         <f>ROWS(Review!J2:J392)-COUNTA(Review!J2:J392)</f>
-        <v>391</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -5012,7 +5057,7 @@
       </c>
       <c r="B12" s="14">
         <f>COUNTIFS(Review!G2:G392,"?*",Review!J2:J392,"")</f>
-        <v>159</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5039,7 +5084,7 @@
     <col min="12" max="12" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5097,7 +5142,9 @@
       <c r="G2" s="3"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="6"/>
+      <c r="J2" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K2" s="7"/>
       <c r="L2" s="7"/>
     </row>
@@ -5121,7 +5168,9 @@
       <c r="G3" s="3"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
-      <c r="J3" s="6"/>
+      <c r="J3" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
     </row>
@@ -5149,7 +5198,9 @@
         <v>24</v>
       </c>
       <c r="I4" s="4"/>
-      <c r="J4" s="6"/>
+      <c r="J4" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
     </row>
@@ -5179,7 +5230,9 @@
         <v>31</v>
       </c>
       <c r="I5" s="4"/>
-      <c r="J5" s="6"/>
+      <c r="J5" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
     </row>
@@ -5203,7 +5256,9 @@
       <c r="G6" s="3"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
-      <c r="J6" s="6"/>
+      <c r="J6" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K6" s="7"/>
       <c r="L6" s="7"/>
     </row>
@@ -5227,7 +5282,9 @@
       <c r="G7" s="3"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
-      <c r="J7" s="6"/>
+      <c r="J7" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
     </row>
@@ -5251,7 +5308,9 @@
       <c r="G8" s="3"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
-      <c r="J8" s="6"/>
+      <c r="J8" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
     </row>
@@ -5275,7 +5334,9 @@
       <c r="G9" s="3"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
-      <c r="J9" s="6"/>
+      <c r="J9" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K9" s="7"/>
       <c r="L9" s="7"/>
     </row>
@@ -5299,7 +5360,9 @@
       <c r="G10" s="3"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
-      <c r="J10" s="6"/>
+      <c r="J10" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
     </row>
@@ -5323,7 +5386,9 @@
       <c r="G11" s="3"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
-      <c r="J11" s="6"/>
+      <c r="J11" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
     </row>
@@ -5347,7 +5412,9 @@
       <c r="G12" s="3"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
-      <c r="J12" s="6"/>
+      <c r="J12" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K12" s="7"/>
       <c r="L12" s="7"/>
     </row>
@@ -5371,7 +5438,9 @@
       <c r="G13" s="3"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="6"/>
+      <c r="J13" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
     </row>
@@ -5395,7 +5464,9 @@
       <c r="G14" s="3"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="6"/>
+      <c r="J14" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
     </row>
@@ -5419,7 +5490,9 @@
       <c r="G15" s="3"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
-      <c r="J15" s="6"/>
+      <c r="J15" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K15" s="7"/>
       <c r="L15" s="7"/>
     </row>
@@ -5443,7 +5516,9 @@
       <c r="G16" s="3"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
-      <c r="J16" s="6"/>
+      <c r="J16" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
     </row>
@@ -5467,7 +5542,9 @@
       <c r="G17" s="3"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
-      <c r="J17" s="6"/>
+      <c r="J17" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
     </row>
@@ -5491,7 +5568,9 @@
       <c r="G18" s="3"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
-      <c r="J18" s="6"/>
+      <c r="J18" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
     </row>
@@ -5515,11 +5594,13 @@
       <c r="G19" s="3"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
-      <c r="J19" s="6"/>
+      <c r="J19" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K19" s="7"/>
       <c r="L19" s="7"/>
     </row>
-    <row r="20" spans="1:12" ht="51" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>12</v>
       </c>
@@ -5543,9 +5624,15 @@
         <v>77</v>
       </c>
       <c r="I20" s="4"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="7"/>
-      <c r="L20" s="7"/>
+      <c r="J20" s="6" t="s">
+        <v>1463</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>1464</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>1465</v>
+      </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
@@ -5567,7 +5654,9 @@
       <c r="G21" s="3"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="6"/>
+      <c r="J21" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K21" s="7"/>
       <c r="L21" s="7"/>
     </row>
@@ -5591,7 +5680,9 @@
       <c r="G22" s="3"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
-      <c r="J22" s="6"/>
+      <c r="J22" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K22" s="7"/>
       <c r="L22" s="7"/>
     </row>
@@ -5615,7 +5706,9 @@
       <c r="G23" s="3"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
-      <c r="J23" s="6"/>
+      <c r="J23" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K23" s="7"/>
       <c r="L23" s="7"/>
     </row>
@@ -5639,7 +5732,9 @@
       <c r="G24" s="3"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
-      <c r="J24" s="6"/>
+      <c r="J24" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K24" s="7"/>
       <c r="L24" s="7"/>
     </row>
@@ -5667,7 +5762,9 @@
         <v>93</v>
       </c>
       <c r="I25" s="4"/>
-      <c r="J25" s="6"/>
+      <c r="J25" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K25" s="7"/>
       <c r="L25" s="7"/>
     </row>
@@ -5691,7 +5788,9 @@
       <c r="G26" s="3"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
-      <c r="J26" s="6"/>
+      <c r="J26" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K26" s="7"/>
       <c r="L26" s="7"/>
     </row>
@@ -5715,7 +5814,9 @@
       <c r="G27" s="3"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
-      <c r="J27" s="6"/>
+      <c r="J27" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K27" s="7"/>
       <c r="L27" s="7"/>
     </row>
@@ -5739,7 +5840,9 @@
       <c r="G28" s="3"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
-      <c r="J28" s="6"/>
+      <c r="J28" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K28" s="7"/>
       <c r="L28" s="7"/>
     </row>
@@ -5767,7 +5870,9 @@
         <v>106</v>
       </c>
       <c r="I29" s="4"/>
-      <c r="J29" s="6"/>
+      <c r="J29" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K29" s="7"/>
       <c r="L29" s="7"/>
     </row>
@@ -5791,7 +5896,9 @@
       <c r="G30" s="3"/>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
-      <c r="J30" s="6"/>
+      <c r="J30" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K30" s="7"/>
       <c r="L30" s="7"/>
     </row>
@@ -5815,7 +5922,9 @@
       <c r="G31" s="3"/>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
-      <c r="J31" s="6"/>
+      <c r="J31" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
     </row>
@@ -5845,7 +5954,9 @@
         <v>31</v>
       </c>
       <c r="I32" s="4"/>
-      <c r="J32" s="6"/>
+      <c r="J32" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K32" s="7"/>
       <c r="L32" s="7"/>
     </row>
@@ -5869,7 +5980,9 @@
       <c r="G33" s="3"/>
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
-      <c r="J33" s="6"/>
+      <c r="J33" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
     </row>
@@ -5893,7 +6006,9 @@
       <c r="G34" s="3"/>
       <c r="H34" s="4"/>
       <c r="I34" s="4"/>
-      <c r="J34" s="6"/>
+      <c r="J34" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K34" s="7"/>
       <c r="L34" s="7"/>
     </row>
@@ -5917,7 +6032,9 @@
       <c r="G35" s="3"/>
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
-      <c r="J35" s="6"/>
+      <c r="J35" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K35" s="7"/>
       <c r="L35" s="7"/>
     </row>
@@ -5941,7 +6058,9 @@
       <c r="G36" s="3"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
-      <c r="J36" s="6"/>
+      <c r="J36" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K36" s="7"/>
       <c r="L36" s="7"/>
     </row>
@@ -5965,7 +6084,9 @@
       <c r="G37" s="3"/>
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
-      <c r="J37" s="6"/>
+      <c r="J37" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K37" s="7"/>
       <c r="L37" s="7"/>
     </row>
@@ -5989,7 +6110,9 @@
       <c r="G38" s="3"/>
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
-      <c r="J38" s="6"/>
+      <c r="J38" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K38" s="7"/>
       <c r="L38" s="7"/>
     </row>
@@ -6013,7 +6136,9 @@
       <c r="G39" s="3"/>
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
-      <c r="J39" s="6"/>
+      <c r="J39" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K39" s="7"/>
       <c r="L39" s="7"/>
     </row>
@@ -6037,7 +6162,9 @@
       <c r="G40" s="3"/>
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
-      <c r="J40" s="6"/>
+      <c r="J40" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K40" s="7"/>
       <c r="L40" s="7"/>
     </row>
@@ -6061,11 +6188,13 @@
       <c r="G41" s="3"/>
       <c r="H41" s="4"/>
       <c r="I41" s="4"/>
-      <c r="J41" s="6"/>
+      <c r="J41" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K41" s="7"/>
       <c r="L41" s="7"/>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:12" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
         <v>12</v>
       </c>
@@ -6085,9 +6214,15 @@
       <c r="G42" s="3"/>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
-      <c r="J42" s="6"/>
-      <c r="K42" s="7"/>
-      <c r="L42" s="7"/>
+      <c r="J42" s="6" t="s">
+        <v>1463</v>
+      </c>
+      <c r="K42" s="7" t="s">
+        <v>1466</v>
+      </c>
+      <c r="L42" s="7" t="s">
+        <v>1467</v>
+      </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
@@ -6109,7 +6244,9 @@
       <c r="G43" s="3"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
-      <c r="J43" s="6"/>
+      <c r="J43" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K43" s="7"/>
       <c r="L43" s="7"/>
     </row>
@@ -6133,7 +6270,9 @@
       <c r="G44" s="3"/>
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
-      <c r="J44" s="6"/>
+      <c r="J44" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K44" s="7"/>
       <c r="L44" s="7"/>
     </row>
@@ -6157,7 +6296,9 @@
       <c r="G45" s="3"/>
       <c r="H45" s="4"/>
       <c r="I45" s="4"/>
-      <c r="J45" s="6"/>
+      <c r="J45" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K45" s="7"/>
       <c r="L45" s="7"/>
     </row>
@@ -6181,7 +6322,9 @@
       <c r="G46" s="3"/>
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
-      <c r="J46" s="6"/>
+      <c r="J46" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K46" s="7"/>
       <c r="L46" s="7"/>
     </row>
@@ -6205,7 +6348,9 @@
       <c r="G47" s="3"/>
       <c r="H47" s="4"/>
       <c r="I47" s="4"/>
-      <c r="J47" s="6"/>
+      <c r="J47" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K47" s="7"/>
       <c r="L47" s="7"/>
     </row>
@@ -6229,7 +6374,9 @@
       <c r="G48" s="3"/>
       <c r="H48" s="4"/>
       <c r="I48" s="4"/>
-      <c r="J48" s="6"/>
+      <c r="J48" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K48" s="7"/>
       <c r="L48" s="7"/>
     </row>
@@ -6253,7 +6400,9 @@
       <c r="G49" s="3"/>
       <c r="H49" s="4"/>
       <c r="I49" s="4"/>
-      <c r="J49" s="6"/>
+      <c r="J49" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K49" s="7"/>
       <c r="L49" s="7"/>
     </row>
@@ -6283,7 +6432,9 @@
         <v>31</v>
       </c>
       <c r="I50" s="4"/>
-      <c r="J50" s="6"/>
+      <c r="J50" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K50" s="7"/>
       <c r="L50" s="7"/>
     </row>
@@ -6307,7 +6458,9 @@
       <c r="G51" s="3"/>
       <c r="H51" s="4"/>
       <c r="I51" s="4"/>
-      <c r="J51" s="6"/>
+      <c r="J51" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K51" s="7"/>
       <c r="L51" s="7"/>
     </row>
@@ -6331,7 +6484,9 @@
       <c r="G52" s="3"/>
       <c r="H52" s="4"/>
       <c r="I52" s="4"/>
-      <c r="J52" s="6"/>
+      <c r="J52" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K52" s="7"/>
       <c r="L52" s="7"/>
     </row>
@@ -6355,7 +6510,9 @@
       <c r="G53" s="3"/>
       <c r="H53" s="4"/>
       <c r="I53" s="4"/>
-      <c r="J53" s="6"/>
+      <c r="J53" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K53" s="7"/>
       <c r="L53" s="7"/>
     </row>
@@ -6379,7 +6536,9 @@
       <c r="G54" s="3"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4"/>
-      <c r="J54" s="6"/>
+      <c r="J54" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K54" s="7"/>
       <c r="L54" s="7"/>
     </row>
@@ -6403,7 +6562,9 @@
       <c r="G55" s="3"/>
       <c r="H55" s="4"/>
       <c r="I55" s="4"/>
-      <c r="J55" s="6"/>
+      <c r="J55" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K55" s="7"/>
       <c r="L55" s="7"/>
     </row>
@@ -6427,7 +6588,9 @@
       <c r="G56" s="3"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4"/>
-      <c r="J56" s="6"/>
+      <c r="J56" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K56" s="7"/>
       <c r="L56" s="7"/>
     </row>
@@ -6451,7 +6614,9 @@
       <c r="G57" s="3"/>
       <c r="H57" s="4"/>
       <c r="I57" s="4"/>
-      <c r="J57" s="6"/>
+      <c r="J57" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K57" s="7"/>
       <c r="L57" s="7"/>
     </row>
@@ -6475,7 +6640,9 @@
       <c r="G58" s="3"/>
       <c r="H58" s="4"/>
       <c r="I58" s="4"/>
-      <c r="J58" s="6"/>
+      <c r="J58" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K58" s="7"/>
       <c r="L58" s="7"/>
     </row>
@@ -6499,7 +6666,9 @@
       <c r="G59" s="3"/>
       <c r="H59" s="4"/>
       <c r="I59" s="4"/>
-      <c r="J59" s="6"/>
+      <c r="J59" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K59" s="7"/>
       <c r="L59" s="7"/>
     </row>
@@ -6523,7 +6692,9 @@
       <c r="G60" s="3"/>
       <c r="H60" s="4"/>
       <c r="I60" s="4"/>
-      <c r="J60" s="6"/>
+      <c r="J60" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K60" s="7"/>
       <c r="L60" s="7"/>
     </row>
@@ -6547,7 +6718,9 @@
       <c r="G61" s="3"/>
       <c r="H61" s="4"/>
       <c r="I61" s="4"/>
-      <c r="J61" s="6"/>
+      <c r="J61" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K61" s="7"/>
       <c r="L61" s="7"/>
     </row>
@@ -6571,7 +6744,9 @@
       <c r="G62" s="3"/>
       <c r="H62" s="4"/>
       <c r="I62" s="4"/>
-      <c r="J62" s="6"/>
+      <c r="J62" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K62" s="7"/>
       <c r="L62" s="7"/>
     </row>
@@ -6595,7 +6770,9 @@
       <c r="G63" s="3"/>
       <c r="H63" s="4"/>
       <c r="I63" s="4"/>
-      <c r="J63" s="6"/>
+      <c r="J63" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K63" s="7"/>
       <c r="L63" s="7"/>
     </row>
@@ -6619,7 +6796,9 @@
       <c r="G64" s="3"/>
       <c r="H64" s="4"/>
       <c r="I64" s="4"/>
-      <c r="J64" s="6"/>
+      <c r="J64" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K64" s="7"/>
       <c r="L64" s="7"/>
     </row>
@@ -6643,7 +6822,9 @@
       <c r="G65" s="3"/>
       <c r="H65" s="4"/>
       <c r="I65" s="4"/>
-      <c r="J65" s="6"/>
+      <c r="J65" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K65" s="7"/>
       <c r="L65" s="7"/>
     </row>
@@ -6667,7 +6848,9 @@
       <c r="G66" s="3"/>
       <c r="H66" s="4"/>
       <c r="I66" s="4"/>
-      <c r="J66" s="6"/>
+      <c r="J66" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K66" s="7"/>
       <c r="L66" s="7"/>
     </row>
@@ -6691,7 +6874,9 @@
       <c r="G67" s="3"/>
       <c r="H67" s="4"/>
       <c r="I67" s="4"/>
-      <c r="J67" s="6"/>
+      <c r="J67" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K67" s="7"/>
       <c r="L67" s="7"/>
     </row>
@@ -6715,7 +6900,9 @@
       <c r="G68" s="3"/>
       <c r="H68" s="4"/>
       <c r="I68" s="4"/>
-      <c r="J68" s="6"/>
+      <c r="J68" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K68" s="7"/>
       <c r="L68" s="7"/>
     </row>
@@ -6739,7 +6926,9 @@
       <c r="G69" s="3"/>
       <c r="H69" s="4"/>
       <c r="I69" s="4"/>
-      <c r="J69" s="6"/>
+      <c r="J69" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K69" s="7"/>
       <c r="L69" s="7"/>
     </row>
@@ -6763,7 +6952,9 @@
       <c r="G70" s="3"/>
       <c r="H70" s="4"/>
       <c r="I70" s="4"/>
-      <c r="J70" s="6"/>
+      <c r="J70" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K70" s="7"/>
       <c r="L70" s="7"/>
     </row>
@@ -6787,7 +6978,9 @@
       <c r="G71" s="3"/>
       <c r="H71" s="4"/>
       <c r="I71" s="4"/>
-      <c r="J71" s="6"/>
+      <c r="J71" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K71" s="7"/>
       <c r="L71" s="7"/>
     </row>
@@ -6811,7 +7004,9 @@
       <c r="G72" s="3"/>
       <c r="H72" s="4"/>
       <c r="I72" s="4"/>
-      <c r="J72" s="6"/>
+      <c r="J72" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K72" s="7"/>
       <c r="L72" s="7"/>
     </row>
@@ -6835,7 +7030,9 @@
       <c r="G73" s="3"/>
       <c r="H73" s="4"/>
       <c r="I73" s="4"/>
-      <c r="J73" s="6"/>
+      <c r="J73" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K73" s="7"/>
       <c r="L73" s="7"/>
     </row>
@@ -6859,7 +7056,9 @@
       <c r="G74" s="3"/>
       <c r="H74" s="4"/>
       <c r="I74" s="4"/>
-      <c r="J74" s="6"/>
+      <c r="J74" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K74" s="7"/>
       <c r="L74" s="7"/>
     </row>
@@ -6883,7 +7082,9 @@
       <c r="G75" s="3"/>
       <c r="H75" s="4"/>
       <c r="I75" s="4"/>
-      <c r="J75" s="6"/>
+      <c r="J75" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K75" s="7"/>
       <c r="L75" s="7"/>
     </row>
@@ -6907,7 +7108,9 @@
       <c r="G76" s="3"/>
       <c r="H76" s="4"/>
       <c r="I76" s="4"/>
-      <c r="J76" s="6"/>
+      <c r="J76" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K76" s="7"/>
       <c r="L76" s="7"/>
     </row>
@@ -6931,7 +7134,9 @@
       <c r="G77" s="3"/>
       <c r="H77" s="4"/>
       <c r="I77" s="4"/>
-      <c r="J77" s="6"/>
+      <c r="J77" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K77" s="7"/>
       <c r="L77" s="7"/>
     </row>
@@ -6955,7 +7160,9 @@
       <c r="G78" s="3"/>
       <c r="H78" s="4"/>
       <c r="I78" s="4"/>
-      <c r="J78" s="6"/>
+      <c r="J78" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K78" s="7"/>
       <c r="L78" s="7"/>
     </row>
@@ -6985,7 +7192,9 @@
         <v>31</v>
       </c>
       <c r="I79" s="4"/>
-      <c r="J79" s="6"/>
+      <c r="J79" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K79" s="7"/>
       <c r="L79" s="7"/>
     </row>
@@ -7009,7 +7218,9 @@
       <c r="G80" s="3"/>
       <c r="H80" s="4"/>
       <c r="I80" s="4"/>
-      <c r="J80" s="6"/>
+      <c r="J80" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K80" s="7"/>
       <c r="L80" s="7"/>
     </row>
@@ -7033,11 +7244,13 @@
       <c r="G81" s="3"/>
       <c r="H81" s="4"/>
       <c r="I81" s="4"/>
-      <c r="J81" s="6"/>
+      <c r="J81" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K81" s="7"/>
       <c r="L81" s="7"/>
     </row>
-    <row r="82" spans="1:12" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:12" ht="51" x14ac:dyDescent="0.2">
       <c r="A82" s="3" t="s">
         <v>12</v>
       </c>
@@ -7061,9 +7274,15 @@
         <v>263</v>
       </c>
       <c r="I82" s="4"/>
-      <c r="J82" s="6"/>
-      <c r="K82" s="7"/>
-      <c r="L82" s="7"/>
+      <c r="J82" s="6" t="s">
+        <v>1463</v>
+      </c>
+      <c r="K82" s="7" t="s">
+        <v>1468</v>
+      </c>
+      <c r="L82" s="7" t="s">
+        <v>1469</v>
+      </c>
     </row>
     <row r="83" spans="1:12" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A83" s="3" t="s">
@@ -7085,7 +7304,9 @@
       <c r="G83" s="3"/>
       <c r="H83" s="4"/>
       <c r="I83" s="4"/>
-      <c r="J83" s="6"/>
+      <c r="J83" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K83" s="7"/>
       <c r="L83" s="7"/>
     </row>
@@ -7109,7 +7330,9 @@
       <c r="G84" s="3"/>
       <c r="H84" s="4"/>
       <c r="I84" s="4"/>
-      <c r="J84" s="6"/>
+      <c r="J84" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K84" s="7"/>
       <c r="L84" s="7"/>
     </row>
@@ -7133,9 +7356,15 @@
       <c r="G85" s="3"/>
       <c r="H85" s="4"/>
       <c r="I85" s="4"/>
-      <c r="J85" s="6"/>
-      <c r="K85" s="7"/>
-      <c r="L85" s="7"/>
+      <c r="J85" s="6" t="s">
+        <v>1463</v>
+      </c>
+      <c r="K85" s="7" t="s">
+        <v>1470</v>
+      </c>
+      <c r="L85" s="7" t="s">
+        <v>1471</v>
+      </c>
     </row>
     <row r="86" spans="1:12" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
@@ -7157,7 +7386,9 @@
       <c r="G86" s="3"/>
       <c r="H86" s="4"/>
       <c r="I86" s="4"/>
-      <c r="J86" s="6"/>
+      <c r="J86" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K86" s="7"/>
       <c r="L86" s="7"/>
     </row>
@@ -7181,7 +7412,9 @@
       <c r="G87" s="3"/>
       <c r="H87" s="4"/>
       <c r="I87" s="4"/>
-      <c r="J87" s="6"/>
+      <c r="J87" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K87" s="7"/>
       <c r="L87" s="7"/>
     </row>
@@ -7205,7 +7438,9 @@
       <c r="G88" s="3"/>
       <c r="H88" s="4"/>
       <c r="I88" s="4"/>
-      <c r="J88" s="6"/>
+      <c r="J88" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K88" s="7"/>
       <c r="L88" s="7"/>
     </row>
@@ -7229,7 +7464,9 @@
       <c r="G89" s="3"/>
       <c r="H89" s="4"/>
       <c r="I89" s="4"/>
-      <c r="J89" s="6"/>
+      <c r="J89" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K89" s="7"/>
       <c r="L89" s="7"/>
     </row>
@@ -7253,7 +7490,9 @@
       <c r="G90" s="3"/>
       <c r="H90" s="4"/>
       <c r="I90" s="4"/>
-      <c r="J90" s="6"/>
+      <c r="J90" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K90" s="7"/>
       <c r="L90" s="7"/>
     </row>
@@ -7277,7 +7516,9 @@
       <c r="G91" s="3"/>
       <c r="H91" s="4"/>
       <c r="I91" s="4"/>
-      <c r="J91" s="6"/>
+      <c r="J91" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K91" s="7"/>
       <c r="L91" s="7"/>
     </row>
@@ -7301,7 +7542,9 @@
       <c r="G92" s="3"/>
       <c r="H92" s="4"/>
       <c r="I92" s="4"/>
-      <c r="J92" s="6"/>
+      <c r="J92" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K92" s="7"/>
       <c r="L92" s="7"/>
     </row>
@@ -7325,7 +7568,9 @@
       <c r="G93" s="3"/>
       <c r="H93" s="4"/>
       <c r="I93" s="4"/>
-      <c r="J93" s="6"/>
+      <c r="J93" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K93" s="7"/>
       <c r="L93" s="7"/>
     </row>
@@ -7349,7 +7594,9 @@
       <c r="G94" s="3"/>
       <c r="H94" s="4"/>
       <c r="I94" s="4"/>
-      <c r="J94" s="6"/>
+      <c r="J94" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K94" s="7"/>
       <c r="L94" s="7"/>
     </row>
@@ -7379,7 +7626,9 @@
         <v>31</v>
       </c>
       <c r="I95" s="4"/>
-      <c r="J95" s="6"/>
+      <c r="J95" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K95" s="7"/>
       <c r="L95" s="7"/>
     </row>
@@ -7403,7 +7652,9 @@
       <c r="G96" s="3"/>
       <c r="H96" s="4"/>
       <c r="I96" s="4"/>
-      <c r="J96" s="6"/>
+      <c r="J96" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K96" s="7"/>
       <c r="L96" s="7"/>
     </row>
@@ -7427,7 +7678,9 @@
       <c r="G97" s="3"/>
       <c r="H97" s="4"/>
       <c r="I97" s="4"/>
-      <c r="J97" s="6"/>
+      <c r="J97" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K97" s="7"/>
       <c r="L97" s="7"/>
     </row>
@@ -7451,7 +7704,9 @@
       <c r="G98" s="3"/>
       <c r="H98" s="4"/>
       <c r="I98" s="4"/>
-      <c r="J98" s="6"/>
+      <c r="J98" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K98" s="7"/>
       <c r="L98" s="7"/>
     </row>
@@ -7475,7 +7730,9 @@
       <c r="G99" s="3"/>
       <c r="H99" s="4"/>
       <c r="I99" s="4"/>
-      <c r="J99" s="6"/>
+      <c r="J99" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K99" s="7"/>
       <c r="L99" s="7"/>
     </row>
@@ -7499,7 +7756,9 @@
       <c r="G100" s="3"/>
       <c r="H100" s="4"/>
       <c r="I100" s="4"/>
-      <c r="J100" s="6"/>
+      <c r="J100" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K100" s="7"/>
       <c r="L100" s="7"/>
     </row>
@@ -7523,7 +7782,9 @@
       <c r="G101" s="3"/>
       <c r="H101" s="4"/>
       <c r="I101" s="4"/>
-      <c r="J101" s="6"/>
+      <c r="J101" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K101" s="7"/>
       <c r="L101" s="7"/>
     </row>
@@ -7547,7 +7808,9 @@
       <c r="G102" s="3"/>
       <c r="H102" s="4"/>
       <c r="I102" s="4"/>
-      <c r="J102" s="6"/>
+      <c r="J102" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K102" s="7"/>
       <c r="L102" s="7"/>
     </row>
@@ -7571,7 +7834,9 @@
       <c r="G103" s="3"/>
       <c r="H103" s="4"/>
       <c r="I103" s="4"/>
-      <c r="J103" s="6"/>
+      <c r="J103" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K103" s="7"/>
       <c r="L103" s="7"/>
     </row>
@@ -7595,7 +7860,9 @@
       <c r="G104" s="3"/>
       <c r="H104" s="4"/>
       <c r="I104" s="4"/>
-      <c r="J104" s="6"/>
+      <c r="J104" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K104" s="7"/>
       <c r="L104" s="7"/>
     </row>
@@ -7619,7 +7886,9 @@
       <c r="G105" s="3"/>
       <c r="H105" s="4"/>
       <c r="I105" s="4"/>
-      <c r="J105" s="6"/>
+      <c r="J105" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K105" s="7"/>
       <c r="L105" s="7"/>
     </row>
@@ -7643,7 +7912,9 @@
       <c r="G106" s="3"/>
       <c r="H106" s="4"/>
       <c r="I106" s="4"/>
-      <c r="J106" s="6"/>
+      <c r="J106" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K106" s="7"/>
       <c r="L106" s="7"/>
     </row>
@@ -7667,7 +7938,9 @@
       <c r="G107" s="3"/>
       <c r="H107" s="4"/>
       <c r="I107" s="4"/>
-      <c r="J107" s="6"/>
+      <c r="J107" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K107" s="7"/>
       <c r="L107" s="7"/>
     </row>
@@ -7691,7 +7964,9 @@
       <c r="G108" s="3"/>
       <c r="H108" s="4"/>
       <c r="I108" s="4"/>
-      <c r="J108" s="6"/>
+      <c r="J108" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K108" s="7"/>
       <c r="L108" s="7"/>
     </row>
@@ -7715,7 +7990,9 @@
       <c r="G109" s="3"/>
       <c r="H109" s="4"/>
       <c r="I109" s="4"/>
-      <c r="J109" s="6"/>
+      <c r="J109" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K109" s="7"/>
       <c r="L109" s="7"/>
     </row>
@@ -7739,7 +8016,9 @@
       <c r="G110" s="3"/>
       <c r="H110" s="4"/>
       <c r="I110" s="4"/>
-      <c r="J110" s="6"/>
+      <c r="J110" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K110" s="7"/>
       <c r="L110" s="7"/>
     </row>
@@ -7763,7 +8042,9 @@
       <c r="G111" s="3"/>
       <c r="H111" s="4"/>
       <c r="I111" s="4"/>
-      <c r="J111" s="6"/>
+      <c r="J111" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K111" s="7"/>
       <c r="L111" s="7"/>
     </row>
@@ -7791,7 +8072,9 @@
         <v>355</v>
       </c>
       <c r="I112" s="4"/>
-      <c r="J112" s="6"/>
+      <c r="J112" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K112" s="7"/>
       <c r="L112" s="7"/>
     </row>
@@ -7815,7 +8098,9 @@
       <c r="G113" s="3"/>
       <c r="H113" s="4"/>
       <c r="I113" s="4"/>
-      <c r="J113" s="6"/>
+      <c r="J113" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K113" s="7"/>
       <c r="L113" s="7"/>
     </row>
@@ -7839,7 +8124,9 @@
       <c r="G114" s="3"/>
       <c r="H114" s="4"/>
       <c r="I114" s="4"/>
-      <c r="J114" s="6"/>
+      <c r="J114" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K114" s="7"/>
       <c r="L114" s="7"/>
     </row>
@@ -7869,7 +8156,9 @@
         <v>366</v>
       </c>
       <c r="I115" s="4"/>
-      <c r="J115" s="6"/>
+      <c r="J115" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K115" s="7"/>
       <c r="L115" s="7"/>
     </row>
@@ -7893,7 +8182,9 @@
       <c r="G116" s="3"/>
       <c r="H116" s="4"/>
       <c r="I116" s="4"/>
-      <c r="J116" s="6"/>
+      <c r="J116" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K116" s="7"/>
       <c r="L116" s="7"/>
     </row>
@@ -7921,7 +8212,9 @@
         <v>373</v>
       </c>
       <c r="I117" s="4"/>
-      <c r="J117" s="6"/>
+      <c r="J117" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K117" s="7"/>
       <c r="L117" s="7"/>
     </row>
@@ -7945,7 +8238,9 @@
       <c r="G118" s="3"/>
       <c r="H118" s="4"/>
       <c r="I118" s="4"/>
-      <c r="J118" s="6"/>
+      <c r="J118" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K118" s="7"/>
       <c r="L118" s="7"/>
     </row>
@@ -7969,7 +8264,9 @@
       <c r="G119" s="3"/>
       <c r="H119" s="4"/>
       <c r="I119" s="4"/>
-      <c r="J119" s="6"/>
+      <c r="J119" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K119" s="7"/>
       <c r="L119" s="7"/>
     </row>
@@ -7997,7 +8294,9 @@
         <v>383</v>
       </c>
       <c r="I120" s="4"/>
-      <c r="J120" s="6"/>
+      <c r="J120" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K120" s="7"/>
       <c r="L120" s="7"/>
     </row>
@@ -8021,7 +8320,9 @@
       <c r="G121" s="3"/>
       <c r="H121" s="4"/>
       <c r="I121" s="4"/>
-      <c r="J121" s="6"/>
+      <c r="J121" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K121" s="7"/>
       <c r="L121" s="7"/>
     </row>
@@ -8045,8 +8346,12 @@
       <c r="G122" s="3"/>
       <c r="H122" s="4"/>
       <c r="I122" s="4"/>
-      <c r="J122" s="6"/>
-      <c r="K122" s="7"/>
+      <c r="J122" s="6" t="s">
+        <v>1463</v>
+      </c>
+      <c r="K122" s="7" t="s">
+        <v>1472</v>
+      </c>
       <c r="L122" s="7"/>
     </row>
     <row r="123" spans="1:12" x14ac:dyDescent="0.2">
@@ -8069,7 +8374,9 @@
       <c r="G123" s="3"/>
       <c r="H123" s="4"/>
       <c r="I123" s="4"/>
-      <c r="J123" s="6"/>
+      <c r="J123" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K123" s="7"/>
       <c r="L123" s="7"/>
     </row>
@@ -8093,7 +8400,9 @@
       <c r="G124" s="3"/>
       <c r="H124" s="4"/>
       <c r="I124" s="4"/>
-      <c r="J124" s="6"/>
+      <c r="J124" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K124" s="7"/>
       <c r="L124" s="7"/>
     </row>
@@ -8117,7 +8426,9 @@
       <c r="G125" s="3"/>
       <c r="H125" s="4"/>
       <c r="I125" s="4"/>
-      <c r="J125" s="6"/>
+      <c r="J125" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K125" s="7"/>
       <c r="L125" s="7"/>
     </row>
@@ -8141,8 +8452,12 @@
       <c r="G126" s="3"/>
       <c r="H126" s="4"/>
       <c r="I126" s="4"/>
-      <c r="J126" s="6"/>
-      <c r="K126" s="7"/>
+      <c r="J126" s="6" t="s">
+        <v>1463</v>
+      </c>
+      <c r="K126" s="7" t="s">
+        <v>1474</v>
+      </c>
       <c r="L126" s="7"/>
     </row>
     <row r="127" spans="1:12" ht="76.5" x14ac:dyDescent="0.2">
@@ -8165,8 +8480,12 @@
       <c r="G127" s="3"/>
       <c r="H127" s="4"/>
       <c r="I127" s="4"/>
-      <c r="J127" s="6"/>
-      <c r="K127" s="7"/>
+      <c r="J127" s="6" t="s">
+        <v>1463</v>
+      </c>
+      <c r="K127" s="7" t="s">
+        <v>1473</v>
+      </c>
       <c r="L127" s="7"/>
     </row>
     <row r="128" spans="1:12" x14ac:dyDescent="0.2">
@@ -8189,8 +8508,12 @@
       <c r="G128" s="3"/>
       <c r="H128" s="4"/>
       <c r="I128" s="4"/>
-      <c r="J128" s="6"/>
-      <c r="K128" s="7"/>
+      <c r="J128" s="6" t="s">
+        <v>1463</v>
+      </c>
+      <c r="K128" s="7" t="s">
+        <v>1475</v>
+      </c>
       <c r="L128" s="7"/>
     </row>
     <row r="129" spans="1:12" ht="63.75" x14ac:dyDescent="0.2">
@@ -8213,7 +8536,9 @@
       <c r="G129" s="3"/>
       <c r="H129" s="4"/>
       <c r="I129" s="4"/>
-      <c r="J129" s="6"/>
+      <c r="J129" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K129" s="7"/>
       <c r="L129" s="7"/>
     </row>
@@ -8237,7 +8562,9 @@
       <c r="G130" s="3"/>
       <c r="H130" s="4"/>
       <c r="I130" s="4"/>
-      <c r="J130" s="6"/>
+      <c r="J130" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K130" s="7"/>
       <c r="L130" s="7"/>
     </row>
@@ -8261,7 +8588,9 @@
       <c r="G131" s="3"/>
       <c r="H131" s="4"/>
       <c r="I131" s="4"/>
-      <c r="J131" s="6"/>
+      <c r="J131" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K131" s="7"/>
       <c r="L131" s="7"/>
     </row>
@@ -8285,7 +8614,9 @@
       <c r="G132" s="3"/>
       <c r="H132" s="4"/>
       <c r="I132" s="4"/>
-      <c r="J132" s="6"/>
+      <c r="J132" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K132" s="7"/>
       <c r="L132" s="7"/>
     </row>
@@ -8309,7 +8640,9 @@
       <c r="G133" s="3"/>
       <c r="H133" s="4"/>
       <c r="I133" s="4"/>
-      <c r="J133" s="6"/>
+      <c r="J133" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K133" s="7"/>
       <c r="L133" s="7"/>
     </row>
@@ -8333,7 +8666,9 @@
       <c r="G134" s="3"/>
       <c r="H134" s="4"/>
       <c r="I134" s="4"/>
-      <c r="J134" s="6"/>
+      <c r="J134" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K134" s="7"/>
       <c r="L134" s="7"/>
     </row>
@@ -8357,7 +8692,9 @@
       <c r="G135" s="3"/>
       <c r="H135" s="4"/>
       <c r="I135" s="4"/>
-      <c r="J135" s="6"/>
+      <c r="J135" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K135" s="7"/>
       <c r="L135" s="7"/>
     </row>
@@ -8381,7 +8718,9 @@
       <c r="G136" s="3"/>
       <c r="H136" s="4"/>
       <c r="I136" s="4"/>
-      <c r="J136" s="6"/>
+      <c r="J136" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K136" s="7"/>
       <c r="L136" s="7"/>
     </row>
@@ -8405,7 +8744,9 @@
       <c r="G137" s="3"/>
       <c r="H137" s="4"/>
       <c r="I137" s="4"/>
-      <c r="J137" s="6"/>
+      <c r="J137" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K137" s="7"/>
       <c r="L137" s="7"/>
     </row>
@@ -8429,7 +8770,9 @@
       <c r="G138" s="3"/>
       <c r="H138" s="4"/>
       <c r="I138" s="4"/>
-      <c r="J138" s="6"/>
+      <c r="J138" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K138" s="7"/>
       <c r="L138" s="7"/>
     </row>
@@ -8453,7 +8796,9 @@
       <c r="G139" s="3"/>
       <c r="H139" s="4"/>
       <c r="I139" s="4"/>
-      <c r="J139" s="6"/>
+      <c r="J139" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K139" s="7"/>
       <c r="L139" s="7"/>
     </row>
@@ -8477,7 +8822,9 @@
       <c r="G140" s="3"/>
       <c r="H140" s="4"/>
       <c r="I140" s="4"/>
-      <c r="J140" s="6"/>
+      <c r="J140" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K140" s="7"/>
       <c r="L140" s="7"/>
     </row>
@@ -8501,7 +8848,9 @@
       <c r="G141" s="3"/>
       <c r="H141" s="4"/>
       <c r="I141" s="4"/>
-      <c r="J141" s="6"/>
+      <c r="J141" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K141" s="7"/>
       <c r="L141" s="7"/>
     </row>
@@ -8525,7 +8874,9 @@
       <c r="G142" s="3"/>
       <c r="H142" s="4"/>
       <c r="I142" s="4"/>
-      <c r="J142" s="6"/>
+      <c r="J142" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K142" s="7"/>
       <c r="L142" s="7"/>
     </row>
@@ -8549,7 +8900,9 @@
       <c r="G143" s="3"/>
       <c r="H143" s="4"/>
       <c r="I143" s="4"/>
-      <c r="J143" s="6"/>
+      <c r="J143" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K143" s="7"/>
       <c r="L143" s="7"/>
     </row>
@@ -8575,7 +8928,9 @@
       <c r="I144" s="10" t="s">
         <v>456</v>
       </c>
-      <c r="J144" s="6"/>
+      <c r="J144" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K144" s="7"/>
       <c r="L144" s="7"/>
     </row>
@@ -8599,7 +8954,9 @@
       <c r="G145" s="3"/>
       <c r="H145" s="4"/>
       <c r="I145" s="4"/>
-      <c r="J145" s="6"/>
+      <c r="J145" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K145" s="7"/>
       <c r="L145" s="7"/>
     </row>
@@ -8623,7 +8980,9 @@
       <c r="G146" s="3"/>
       <c r="H146" s="4"/>
       <c r="I146" s="4"/>
-      <c r="J146" s="6"/>
+      <c r="J146" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K146" s="7"/>
       <c r="L146" s="7"/>
     </row>
@@ -8651,7 +9010,9 @@
         <v>466</v>
       </c>
       <c r="I147" s="4"/>
-      <c r="J147" s="6"/>
+      <c r="J147" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K147" s="7"/>
       <c r="L147" s="7"/>
     </row>
@@ -8679,7 +9040,9 @@
         <v>470</v>
       </c>
       <c r="I148" s="4"/>
-      <c r="J148" s="6"/>
+      <c r="J148" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K148" s="7"/>
       <c r="L148" s="7"/>
     </row>
@@ -8707,7 +9070,9 @@
         <v>470</v>
       </c>
       <c r="I149" s="4"/>
-      <c r="J149" s="6"/>
+      <c r="J149" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K149" s="7"/>
       <c r="L149" s="7"/>
     </row>
@@ -8735,7 +9100,9 @@
         <v>477</v>
       </c>
       <c r="I150" s="4"/>
-      <c r="J150" s="6"/>
+      <c r="J150" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K150" s="7"/>
       <c r="L150" s="7"/>
     </row>
@@ -8759,7 +9126,9 @@
       <c r="G151" s="3"/>
       <c r="H151" s="4"/>
       <c r="I151" s="4"/>
-      <c r="J151" s="6"/>
+      <c r="J151" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K151" s="7"/>
       <c r="L151" s="7"/>
     </row>
@@ -8783,7 +9152,9 @@
       <c r="G152" s="3"/>
       <c r="H152" s="4"/>
       <c r="I152" s="4"/>
-      <c r="J152" s="6"/>
+      <c r="J152" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K152" s="7"/>
       <c r="L152" s="7"/>
     </row>
@@ -8807,7 +9178,9 @@
       <c r="G153" s="3"/>
       <c r="H153" s="4"/>
       <c r="I153" s="4"/>
-      <c r="J153" s="6"/>
+      <c r="J153" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K153" s="7"/>
       <c r="L153" s="7"/>
     </row>
@@ -8831,7 +9204,9 @@
       <c r="G154" s="3"/>
       <c r="H154" s="4"/>
       <c r="I154" s="4"/>
-      <c r="J154" s="6"/>
+      <c r="J154" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K154" s="7"/>
       <c r="L154" s="7"/>
     </row>
@@ -8859,7 +9234,9 @@
         <v>492</v>
       </c>
       <c r="I155" s="4"/>
-      <c r="J155" s="6"/>
+      <c r="J155" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K155" s="7"/>
       <c r="L155" s="7"/>
     </row>
@@ -8883,7 +9260,9 @@
       <c r="G156" s="3"/>
       <c r="H156" s="4"/>
       <c r="I156" s="4"/>
-      <c r="J156" s="6"/>
+      <c r="J156" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K156" s="7"/>
       <c r="L156" s="7"/>
     </row>
@@ -8907,7 +9286,9 @@
       <c r="G157" s="3"/>
       <c r="H157" s="4"/>
       <c r="I157" s="4"/>
-      <c r="J157" s="6"/>
+      <c r="J157" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K157" s="7"/>
       <c r="L157" s="7"/>
     </row>
@@ -8931,7 +9312,9 @@
       <c r="G158" s="3"/>
       <c r="H158" s="4"/>
       <c r="I158" s="4"/>
-      <c r="J158" s="6"/>
+      <c r="J158" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K158" s="7"/>
       <c r="L158" s="7"/>
     </row>
@@ -8955,7 +9338,9 @@
       <c r="G159" s="3"/>
       <c r="H159" s="4"/>
       <c r="I159" s="4"/>
-      <c r="J159" s="6"/>
+      <c r="J159" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K159" s="7"/>
       <c r="L159" s="7"/>
     </row>
@@ -8979,7 +9364,9 @@
       <c r="G160" s="3"/>
       <c r="H160" s="4"/>
       <c r="I160" s="4"/>
-      <c r="J160" s="6"/>
+      <c r="J160" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K160" s="7"/>
       <c r="L160" s="7"/>
     </row>
@@ -9003,7 +9390,9 @@
       <c r="G161" s="3"/>
       <c r="H161" s="4"/>
       <c r="I161" s="4"/>
-      <c r="J161" s="6"/>
+      <c r="J161" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K161" s="7"/>
       <c r="L161" s="7"/>
     </row>
@@ -9027,7 +9416,9 @@
       <c r="G162" s="3"/>
       <c r="H162" s="4"/>
       <c r="I162" s="4"/>
-      <c r="J162" s="6"/>
+      <c r="J162" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K162" s="7"/>
       <c r="L162" s="7"/>
     </row>
@@ -9051,7 +9442,9 @@
       <c r="G163" s="3"/>
       <c r="H163" s="4"/>
       <c r="I163" s="4"/>
-      <c r="J163" s="6"/>
+      <c r="J163" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K163" s="7"/>
       <c r="L163" s="7"/>
     </row>
@@ -9075,7 +9468,9 @@
       <c r="G164" s="3"/>
       <c r="H164" s="4"/>
       <c r="I164" s="4"/>
-      <c r="J164" s="6"/>
+      <c r="J164" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K164" s="7"/>
       <c r="L164" s="7"/>
     </row>
@@ -9099,7 +9494,9 @@
       <c r="G165" s="3"/>
       <c r="H165" s="4"/>
       <c r="I165" s="4"/>
-      <c r="J165" s="6"/>
+      <c r="J165" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K165" s="7"/>
       <c r="L165" s="7"/>
     </row>
@@ -9123,7 +9520,9 @@
       <c r="G166" s="3"/>
       <c r="H166" s="4"/>
       <c r="I166" s="4"/>
-      <c r="J166" s="6"/>
+      <c r="J166" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K166" s="7"/>
       <c r="L166" s="7"/>
     </row>
@@ -9147,7 +9546,9 @@
       <c r="G167" s="3"/>
       <c r="H167" s="4"/>
       <c r="I167" s="4"/>
-      <c r="J167" s="6"/>
+      <c r="J167" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K167" s="7"/>
       <c r="L167" s="7"/>
     </row>
@@ -9171,7 +9572,9 @@
       <c r="G168" s="3"/>
       <c r="H168" s="4"/>
       <c r="I168" s="4"/>
-      <c r="J168" s="6"/>
+      <c r="J168" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K168" s="7"/>
       <c r="L168" s="7"/>
     </row>
@@ -9197,7 +9600,9 @@
       <c r="I169" s="10" t="s">
         <v>535</v>
       </c>
-      <c r="J169" s="6"/>
+      <c r="J169" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K169" s="7"/>
       <c r="L169" s="7"/>
     </row>
@@ -9221,7 +9626,9 @@
       <c r="G170" s="3"/>
       <c r="H170" s="4"/>
       <c r="I170" s="4"/>
-      <c r="J170" s="6"/>
+      <c r="J170" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K170" s="7"/>
       <c r="L170" s="7"/>
     </row>
@@ -9245,7 +9652,9 @@
       <c r="G171" s="3"/>
       <c r="H171" s="4"/>
       <c r="I171" s="4"/>
-      <c r="J171" s="6"/>
+      <c r="J171" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K171" s="7"/>
       <c r="L171" s="7"/>
     </row>
@@ -9269,7 +9678,9 @@
       <c r="G172" s="3"/>
       <c r="H172" s="4"/>
       <c r="I172" s="4"/>
-      <c r="J172" s="6"/>
+      <c r="J172" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K172" s="7"/>
       <c r="L172" s="7"/>
     </row>
@@ -9293,7 +9704,9 @@
       <c r="G173" s="3"/>
       <c r="H173" s="4"/>
       <c r="I173" s="4"/>
-      <c r="J173" s="6"/>
+      <c r="J173" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K173" s="7"/>
       <c r="L173" s="7"/>
     </row>
@@ -9317,7 +9730,9 @@
       <c r="G174" s="3"/>
       <c r="H174" s="4"/>
       <c r="I174" s="4"/>
-      <c r="J174" s="6"/>
+      <c r="J174" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K174" s="7"/>
       <c r="L174" s="7"/>
     </row>
@@ -9341,7 +9756,9 @@
       <c r="G175" s="3"/>
       <c r="H175" s="4"/>
       <c r="I175" s="4"/>
-      <c r="J175" s="6"/>
+      <c r="J175" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K175" s="7"/>
       <c r="L175" s="7"/>
     </row>
@@ -9365,7 +9782,9 @@
       <c r="G176" s="3"/>
       <c r="H176" s="4"/>
       <c r="I176" s="4"/>
-      <c r="J176" s="6"/>
+      <c r="J176" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K176" s="7"/>
       <c r="L176" s="7"/>
     </row>
@@ -9389,7 +9808,9 @@
       <c r="G177" s="3"/>
       <c r="H177" s="4"/>
       <c r="I177" s="4"/>
-      <c r="J177" s="6"/>
+      <c r="J177" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K177" s="7"/>
       <c r="L177" s="7"/>
     </row>
@@ -9413,7 +9834,9 @@
       <c r="G178" s="3"/>
       <c r="H178" s="4"/>
       <c r="I178" s="4"/>
-      <c r="J178" s="6"/>
+      <c r="J178" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K178" s="7"/>
       <c r="L178" s="7"/>
     </row>
@@ -9437,7 +9860,9 @@
       <c r="G179" s="3"/>
       <c r="H179" s="4"/>
       <c r="I179" s="4"/>
-      <c r="J179" s="6"/>
+      <c r="J179" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K179" s="7"/>
       <c r="L179" s="7"/>
     </row>
@@ -9461,7 +9886,9 @@
       <c r="G180" s="3"/>
       <c r="H180" s="4"/>
       <c r="I180" s="4"/>
-      <c r="J180" s="6"/>
+      <c r="J180" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K180" s="7"/>
       <c r="L180" s="7"/>
     </row>
@@ -9485,7 +9912,9 @@
       <c r="G181" s="3"/>
       <c r="H181" s="4"/>
       <c r="I181" s="4"/>
-      <c r="J181" s="6"/>
+      <c r="J181" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K181" s="7"/>
       <c r="L181" s="7"/>
     </row>
@@ -9509,7 +9938,9 @@
       <c r="G182" s="3"/>
       <c r="H182" s="4"/>
       <c r="I182" s="4"/>
-      <c r="J182" s="6"/>
+      <c r="J182" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K182" s="7"/>
       <c r="L182" s="7"/>
     </row>
@@ -9533,7 +9964,9 @@
       <c r="G183" s="3"/>
       <c r="H183" s="4"/>
       <c r="I183" s="4"/>
-      <c r="J183" s="6"/>
+      <c r="J183" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K183" s="7"/>
       <c r="L183" s="7"/>
     </row>
@@ -9557,7 +9990,9 @@
       <c r="G184" s="3"/>
       <c r="H184" s="4"/>
       <c r="I184" s="4"/>
-      <c r="J184" s="6"/>
+      <c r="J184" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K184" s="7"/>
       <c r="L184" s="7"/>
     </row>
@@ -9581,7 +10016,9 @@
       <c r="G185" s="3"/>
       <c r="H185" s="4"/>
       <c r="I185" s="4"/>
-      <c r="J185" s="6"/>
+      <c r="J185" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K185" s="7"/>
       <c r="L185" s="7"/>
     </row>
@@ -9605,7 +10042,9 @@
       <c r="G186" s="3"/>
       <c r="H186" s="4"/>
       <c r="I186" s="4"/>
-      <c r="J186" s="6"/>
+      <c r="J186" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K186" s="7"/>
       <c r="L186" s="7"/>
     </row>
@@ -9629,7 +10068,9 @@
       <c r="G187" s="3"/>
       <c r="H187" s="4"/>
       <c r="I187" s="4"/>
-      <c r="J187" s="6"/>
+      <c r="J187" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K187" s="7"/>
       <c r="L187" s="7"/>
     </row>
@@ -9653,7 +10094,9 @@
       <c r="G188" s="3"/>
       <c r="H188" s="4"/>
       <c r="I188" s="4"/>
-      <c r="J188" s="6"/>
+      <c r="J188" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K188" s="7"/>
       <c r="L188" s="7"/>
     </row>
@@ -9677,7 +10120,9 @@
       <c r="G189" s="3"/>
       <c r="H189" s="4"/>
       <c r="I189" s="4"/>
-      <c r="J189" s="6"/>
+      <c r="J189" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K189" s="7"/>
       <c r="L189" s="7"/>
     </row>
@@ -9701,7 +10146,9 @@
       <c r="G190" s="3"/>
       <c r="H190" s="4"/>
       <c r="I190" s="4"/>
-      <c r="J190" s="6"/>
+      <c r="J190" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K190" s="7"/>
       <c r="L190" s="7"/>
     </row>
@@ -9725,7 +10172,9 @@
       <c r="G191" s="3"/>
       <c r="H191" s="4"/>
       <c r="I191" s="4"/>
-      <c r="J191" s="6"/>
+      <c r="J191" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K191" s="7"/>
       <c r="L191" s="7"/>
     </row>
@@ -9749,7 +10198,9 @@
       <c r="G192" s="3"/>
       <c r="H192" s="4"/>
       <c r="I192" s="4"/>
-      <c r="J192" s="6"/>
+      <c r="J192" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K192" s="7"/>
       <c r="L192" s="7"/>
     </row>
@@ -9773,7 +10224,9 @@
       <c r="G193" s="3"/>
       <c r="H193" s="4"/>
       <c r="I193" s="4"/>
-      <c r="J193" s="6"/>
+      <c r="J193" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K193" s="7"/>
       <c r="L193" s="7"/>
     </row>
@@ -9803,7 +10256,9 @@
         <v>612</v>
       </c>
       <c r="I194" s="4"/>
-      <c r="J194" s="6"/>
+      <c r="J194" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K194" s="7"/>
       <c r="L194" s="7"/>
     </row>
@@ -9833,7 +10288,9 @@
         <v>617</v>
       </c>
       <c r="I195" s="4"/>
-      <c r="J195" s="6"/>
+      <c r="J195" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K195" s="7"/>
       <c r="L195" s="7"/>
     </row>
@@ -9863,7 +10320,9 @@
         <v>622</v>
       </c>
       <c r="I196" s="4"/>
-      <c r="J196" s="6"/>
+      <c r="J196" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K196" s="7"/>
       <c r="L196" s="7"/>
     </row>
@@ -9893,7 +10352,9 @@
         <v>470</v>
       </c>
       <c r="I197" s="4"/>
-      <c r="J197" s="6"/>
+      <c r="J197" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K197" s="7"/>
       <c r="L197" s="7"/>
     </row>
@@ -9923,7 +10384,9 @@
         <v>470</v>
       </c>
       <c r="I198" s="4"/>
-      <c r="J198" s="6"/>
+      <c r="J198" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K198" s="7"/>
       <c r="L198" s="7"/>
     </row>
@@ -9953,7 +10416,9 @@
         <v>633</v>
       </c>
       <c r="I199" s="4"/>
-      <c r="J199" s="6"/>
+      <c r="J199" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K199" s="7"/>
       <c r="L199" s="7"/>
     </row>
@@ -9983,7 +10448,9 @@
         <v>638</v>
       </c>
       <c r="I200" s="4"/>
-      <c r="J200" s="6"/>
+      <c r="J200" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K200" s="7"/>
       <c r="L200" s="7"/>
     </row>
@@ -10013,7 +10480,9 @@
         <v>643</v>
       </c>
       <c r="I201" s="4"/>
-      <c r="J201" s="6"/>
+      <c r="J201" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K201" s="7"/>
       <c r="L201" s="7"/>
     </row>
@@ -10043,7 +10512,9 @@
         <v>648</v>
       </c>
       <c r="I202" s="4"/>
-      <c r="J202" s="6"/>
+      <c r="J202" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K202" s="7"/>
       <c r="L202" s="7"/>
     </row>
@@ -10073,7 +10544,9 @@
         <v>653</v>
       </c>
       <c r="I203" s="4"/>
-      <c r="J203" s="6"/>
+      <c r="J203" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K203" s="7"/>
       <c r="L203" s="7"/>
     </row>
@@ -10103,7 +10576,9 @@
         <v>638</v>
       </c>
       <c r="I204" s="4"/>
-      <c r="J204" s="6"/>
+      <c r="J204" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K204" s="7"/>
       <c r="L204" s="7"/>
     </row>
@@ -10127,7 +10602,9 @@
       <c r="G205" s="3"/>
       <c r="H205" s="4"/>
       <c r="I205" s="4"/>
-      <c r="J205" s="6"/>
+      <c r="J205" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K205" s="7"/>
       <c r="L205" s="7"/>
     </row>
@@ -10155,7 +10632,9 @@
       <c r="I206" s="10" t="s">
         <v>665</v>
       </c>
-      <c r="J206" s="6"/>
+      <c r="J206" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K206" s="7"/>
       <c r="L206" s="7"/>
     </row>
@@ -10185,7 +10664,9 @@
         <v>670</v>
       </c>
       <c r="I207" s="4"/>
-      <c r="J207" s="6"/>
+      <c r="J207" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K207" s="7"/>
       <c r="L207" s="7"/>
     </row>
@@ -10215,7 +10696,9 @@
         <v>470</v>
       </c>
       <c r="I208" s="4"/>
-      <c r="J208" s="6"/>
+      <c r="J208" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K208" s="7"/>
       <c r="L208" s="7"/>
     </row>
@@ -10245,7 +10728,9 @@
         <v>470</v>
       </c>
       <c r="I209" s="4"/>
-      <c r="J209" s="6"/>
+      <c r="J209" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K209" s="7"/>
       <c r="L209" s="7"/>
     </row>
@@ -10275,7 +10760,9 @@
         <v>680</v>
       </c>
       <c r="I210" s="4"/>
-      <c r="J210" s="6"/>
+      <c r="J210" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K210" s="7"/>
       <c r="L210" s="7"/>
     </row>
@@ -10301,7 +10788,9 @@
       <c r="G211" s="3"/>
       <c r="H211" s="4"/>
       <c r="I211" s="4"/>
-      <c r="J211" s="6"/>
+      <c r="J211" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K211" s="7"/>
       <c r="L211" s="7"/>
     </row>
@@ -10331,7 +10820,9 @@
         <v>688</v>
       </c>
       <c r="I212" s="4"/>
-      <c r="J212" s="6"/>
+      <c r="J212" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K212" s="7"/>
       <c r="L212" s="7"/>
     </row>
@@ -10357,7 +10848,9 @@
       <c r="G213" s="3"/>
       <c r="H213" s="4"/>
       <c r="I213" s="4"/>
-      <c r="J213" s="6"/>
+      <c r="J213" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K213" s="7"/>
       <c r="L213" s="7"/>
     </row>
@@ -10387,7 +10880,9 @@
         <v>696</v>
       </c>
       <c r="I214" s="4"/>
-      <c r="J214" s="6"/>
+      <c r="J214" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K214" s="7"/>
       <c r="L214" s="7"/>
     </row>
@@ -10413,7 +10908,9 @@
       <c r="G215" s="3"/>
       <c r="H215" s="4"/>
       <c r="I215" s="4"/>
-      <c r="J215" s="6"/>
+      <c r="J215" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K215" s="7"/>
       <c r="L215" s="7"/>
     </row>
@@ -10443,7 +10940,9 @@
         <v>704</v>
       </c>
       <c r="I216" s="4"/>
-      <c r="J216" s="6"/>
+      <c r="J216" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K216" s="7"/>
       <c r="L216" s="7"/>
     </row>
@@ -10473,7 +10972,9 @@
         <v>470</v>
       </c>
       <c r="I217" s="4"/>
-      <c r="J217" s="6"/>
+      <c r="J217" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K217" s="7"/>
       <c r="L217" s="7"/>
     </row>
@@ -10499,7 +11000,9 @@
       <c r="G218" s="3"/>
       <c r="H218" s="4"/>
       <c r="I218" s="4"/>
-      <c r="J218" s="6"/>
+      <c r="J218" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K218" s="7"/>
       <c r="L218" s="7"/>
     </row>
@@ -10529,7 +11032,9 @@
         <v>715</v>
       </c>
       <c r="I219" s="4"/>
-      <c r="J219" s="6"/>
+      <c r="J219" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K219" s="7"/>
       <c r="L219" s="7"/>
     </row>
@@ -10555,7 +11060,9 @@
       <c r="G220" s="3"/>
       <c r="H220" s="4"/>
       <c r="I220" s="4"/>
-      <c r="J220" s="6"/>
+      <c r="J220" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K220" s="7"/>
       <c r="L220" s="7"/>
     </row>
@@ -10585,7 +11092,9 @@
         <v>723</v>
       </c>
       <c r="I221" s="4"/>
-      <c r="J221" s="6"/>
+      <c r="J221" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K221" s="7"/>
       <c r="L221" s="7"/>
     </row>
@@ -10615,7 +11124,9 @@
         <v>728</v>
       </c>
       <c r="I222" s="4"/>
-      <c r="J222" s="6"/>
+      <c r="J222" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K222" s="7"/>
       <c r="L222" s="7"/>
     </row>
@@ -10641,7 +11152,9 @@
       <c r="G223" s="3"/>
       <c r="H223" s="4"/>
       <c r="I223" s="4"/>
-      <c r="J223" s="6"/>
+      <c r="J223" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K223" s="7"/>
       <c r="L223" s="7"/>
     </row>
@@ -10671,7 +11184,9 @@
         <v>736</v>
       </c>
       <c r="I224" s="4"/>
-      <c r="J224" s="6"/>
+      <c r="J224" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K224" s="7"/>
       <c r="L224" s="7"/>
     </row>
@@ -10695,7 +11210,9 @@
       <c r="G225" s="3"/>
       <c r="H225" s="4"/>
       <c r="I225" s="4"/>
-      <c r="J225" s="6"/>
+      <c r="J225" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K225" s="7"/>
       <c r="L225" s="7"/>
     </row>
@@ -10725,7 +11242,9 @@
         <v>744</v>
       </c>
       <c r="I226" s="4"/>
-      <c r="J226" s="6"/>
+      <c r="J226" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K226" s="7"/>
       <c r="L226" s="7"/>
     </row>
@@ -10755,7 +11274,9 @@
         <v>748</v>
       </c>
       <c r="I227" s="4"/>
-      <c r="J227" s="6"/>
+      <c r="J227" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K227" s="7"/>
       <c r="L227" s="7"/>
     </row>
@@ -10785,7 +11306,9 @@
         <v>753</v>
       </c>
       <c r="I228" s="4"/>
-      <c r="J228" s="6"/>
+      <c r="J228" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K228" s="7"/>
       <c r="L228" s="7"/>
     </row>
@@ -10815,7 +11338,9 @@
         <v>758</v>
       </c>
       <c r="I229" s="4"/>
-      <c r="J229" s="6"/>
+      <c r="J229" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K229" s="7"/>
       <c r="L229" s="7"/>
     </row>
@@ -10841,7 +11366,9 @@
       <c r="G230" s="3"/>
       <c r="H230" s="4"/>
       <c r="I230" s="4"/>
-      <c r="J230" s="6"/>
+      <c r="J230" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K230" s="7"/>
       <c r="L230" s="7"/>
     </row>
@@ -10871,7 +11398,9 @@
         <v>704</v>
       </c>
       <c r="I231" s="4"/>
-      <c r="J231" s="6"/>
+      <c r="J231" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K231" s="7"/>
       <c r="L231" s="7"/>
     </row>
@@ -10901,7 +11430,9 @@
         <v>770</v>
       </c>
       <c r="I232" s="4"/>
-      <c r="J232" s="6"/>
+      <c r="J232" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K232" s="7"/>
       <c r="L232" s="7"/>
     </row>
@@ -10931,7 +11462,9 @@
         <v>775</v>
       </c>
       <c r="I233" s="4"/>
-      <c r="J233" s="6"/>
+      <c r="J233" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K233" s="7"/>
       <c r="L233" s="7"/>
     </row>
@@ -10957,7 +11490,9 @@
       <c r="G234" s="3"/>
       <c r="H234" s="4"/>
       <c r="I234" s="4"/>
-      <c r="J234" s="6"/>
+      <c r="J234" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K234" s="7"/>
       <c r="L234" s="7"/>
     </row>
@@ -10987,7 +11522,9 @@
         <v>783</v>
       </c>
       <c r="I235" s="4"/>
-      <c r="J235" s="6"/>
+      <c r="J235" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K235" s="7"/>
       <c r="L235" s="7"/>
     </row>
@@ -11019,7 +11556,9 @@
       <c r="I236" s="10" t="s">
         <v>789</v>
       </c>
-      <c r="J236" s="6"/>
+      <c r="J236" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K236" s="7"/>
       <c r="L236" s="7"/>
     </row>
@@ -11049,7 +11588,9 @@
         <v>794</v>
       </c>
       <c r="I237" s="4"/>
-      <c r="J237" s="6"/>
+      <c r="J237" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K237" s="7"/>
       <c r="L237" s="7"/>
     </row>
@@ -11079,7 +11620,9 @@
         <v>470</v>
       </c>
       <c r="I238" s="4"/>
-      <c r="J238" s="6"/>
+      <c r="J238" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K238" s="7"/>
       <c r="L238" s="7"/>
     </row>
@@ -11109,7 +11652,9 @@
         <v>803</v>
       </c>
       <c r="I239" s="4"/>
-      <c r="J239" s="6"/>
+      <c r="J239" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K239" s="7"/>
       <c r="L239" s="7"/>
     </row>
@@ -11139,7 +11684,9 @@
         <v>638</v>
       </c>
       <c r="I240" s="4"/>
-      <c r="J240" s="6"/>
+      <c r="J240" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K240" s="7"/>
       <c r="L240" s="7"/>
     </row>
@@ -11169,7 +11716,9 @@
         <v>812</v>
       </c>
       <c r="I241" s="4"/>
-      <c r="J241" s="6"/>
+      <c r="J241" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K241" s="7"/>
       <c r="L241" s="7"/>
     </row>
@@ -11195,7 +11744,9 @@
       <c r="G242" s="3"/>
       <c r="H242" s="4"/>
       <c r="I242" s="4"/>
-      <c r="J242" s="6"/>
+      <c r="J242" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K242" s="7"/>
       <c r="L242" s="7"/>
     </row>
@@ -11225,7 +11776,9 @@
         <v>820</v>
       </c>
       <c r="I243" s="4"/>
-      <c r="J243" s="6"/>
+      <c r="J243" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K243" s="7"/>
       <c r="L243" s="7"/>
     </row>
@@ -11251,7 +11804,9 @@
       <c r="G244" s="3"/>
       <c r="H244" s="4"/>
       <c r="I244" s="4"/>
-      <c r="J244" s="6"/>
+      <c r="J244" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K244" s="7"/>
       <c r="L244" s="7"/>
     </row>
@@ -11281,7 +11836,9 @@
         <v>828</v>
       </c>
       <c r="I245" s="4"/>
-      <c r="J245" s="6"/>
+      <c r="J245" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K245" s="7"/>
       <c r="L245" s="7"/>
     </row>
@@ -11307,7 +11864,9 @@
       <c r="G246" s="3"/>
       <c r="H246" s="4"/>
       <c r="I246" s="4"/>
-      <c r="J246" s="6"/>
+      <c r="J246" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K246" s="7"/>
       <c r="L246" s="7"/>
     </row>
@@ -11337,7 +11896,9 @@
         <v>836</v>
       </c>
       <c r="I247" s="4"/>
-      <c r="J247" s="6"/>
+      <c r="J247" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K247" s="7"/>
       <c r="L247" s="7"/>
     </row>
@@ -11363,7 +11924,9 @@
       <c r="G248" s="3"/>
       <c r="H248" s="4"/>
       <c r="I248" s="4"/>
-      <c r="J248" s="6"/>
+      <c r="J248" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K248" s="7"/>
       <c r="L248" s="7"/>
     </row>
@@ -11393,7 +11956,9 @@
         <v>844</v>
       </c>
       <c r="I249" s="4"/>
-      <c r="J249" s="6"/>
+      <c r="J249" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K249" s="7"/>
       <c r="L249" s="7"/>
     </row>
@@ -11423,7 +11988,9 @@
         <v>470</v>
       </c>
       <c r="I250" s="4"/>
-      <c r="J250" s="6"/>
+      <c r="J250" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K250" s="7"/>
       <c r="L250" s="7"/>
     </row>
@@ -11453,7 +12020,9 @@
         <v>758</v>
       </c>
       <c r="I251" s="4"/>
-      <c r="J251" s="6"/>
+      <c r="J251" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K251" s="7"/>
       <c r="L251" s="7"/>
     </row>
@@ -11483,7 +12052,9 @@
         <v>857</v>
       </c>
       <c r="I252" s="4"/>
-      <c r="J252" s="6"/>
+      <c r="J252" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K252" s="7"/>
       <c r="L252" s="7"/>
     </row>
@@ -11513,7 +12084,9 @@
         <v>862</v>
       </c>
       <c r="I253" s="4"/>
-      <c r="J253" s="6"/>
+      <c r="J253" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K253" s="7"/>
       <c r="L253" s="7"/>
     </row>
@@ -11537,7 +12110,9 @@
       <c r="G254" s="3"/>
       <c r="H254" s="4"/>
       <c r="I254" s="4"/>
-      <c r="J254" s="6"/>
+      <c r="J254" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K254" s="7"/>
       <c r="L254" s="7"/>
     </row>
@@ -11567,7 +12142,9 @@
         <v>870</v>
       </c>
       <c r="I255" s="4"/>
-      <c r="J255" s="6"/>
+      <c r="J255" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K255" s="7"/>
       <c r="L255" s="7"/>
     </row>
@@ -11597,7 +12174,9 @@
         <v>870</v>
       </c>
       <c r="I256" s="4"/>
-      <c r="J256" s="6"/>
+      <c r="J256" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K256" s="7"/>
       <c r="L256" s="7"/>
     </row>
@@ -11629,7 +12208,9 @@
       <c r="I257" s="10" t="s">
         <v>880</v>
       </c>
-      <c r="J257" s="6"/>
+      <c r="J257" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K257" s="7"/>
       <c r="L257" s="7"/>
     </row>
@@ -11661,7 +12242,9 @@
       <c r="I258" s="10" t="s">
         <v>880</v>
       </c>
-      <c r="J258" s="6"/>
+      <c r="J258" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K258" s="7"/>
       <c r="L258" s="7"/>
     </row>
@@ -11685,7 +12268,9 @@
       <c r="G259" s="3"/>
       <c r="H259" s="4"/>
       <c r="I259" s="4"/>
-      <c r="J259" s="6"/>
+      <c r="J259" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K259" s="7"/>
       <c r="L259" s="7"/>
     </row>
@@ -11709,7 +12294,9 @@
       <c r="G260" s="3"/>
       <c r="H260" s="4"/>
       <c r="I260" s="4"/>
-      <c r="J260" s="6"/>
+      <c r="J260" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K260" s="7"/>
       <c r="L260" s="7"/>
     </row>
@@ -11733,7 +12320,9 @@
       <c r="G261" s="3"/>
       <c r="H261" s="4"/>
       <c r="I261" s="4"/>
-      <c r="J261" s="6"/>
+      <c r="J261" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K261" s="7"/>
       <c r="L261" s="7"/>
     </row>
@@ -11757,7 +12346,9 @@
       <c r="G262" s="3"/>
       <c r="H262" s="4"/>
       <c r="I262" s="4"/>
-      <c r="J262" s="6"/>
+      <c r="J262" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K262" s="7"/>
       <c r="L262" s="7"/>
     </row>
@@ -11787,7 +12378,9 @@
         <v>901</v>
       </c>
       <c r="I263" s="4"/>
-      <c r="J263" s="6"/>
+      <c r="J263" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K263" s="7"/>
       <c r="L263" s="7"/>
     </row>
@@ -11811,7 +12404,9 @@
       <c r="G264" s="3"/>
       <c r="H264" s="4"/>
       <c r="I264" s="4"/>
-      <c r="J264" s="6"/>
+      <c r="J264" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K264" s="7"/>
       <c r="L264" s="7"/>
     </row>
@@ -11841,7 +12436,9 @@
         <v>909</v>
       </c>
       <c r="I265" s="4"/>
-      <c r="J265" s="6"/>
+      <c r="J265" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K265" s="7"/>
       <c r="L265" s="7"/>
     </row>
@@ -11865,7 +12462,9 @@
       <c r="G266" s="3"/>
       <c r="H266" s="4"/>
       <c r="I266" s="4"/>
-      <c r="J266" s="6"/>
+      <c r="J266" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K266" s="7"/>
       <c r="L266" s="7"/>
     </row>
@@ -11895,7 +12494,9 @@
         <v>916</v>
       </c>
       <c r="I267" s="4"/>
-      <c r="J267" s="6"/>
+      <c r="J267" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K267" s="7"/>
       <c r="L267" s="7"/>
     </row>
@@ -11919,7 +12520,9 @@
       <c r="G268" s="3"/>
       <c r="H268" s="4"/>
       <c r="I268" s="4"/>
-      <c r="J268" s="6"/>
+      <c r="J268" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K268" s="7"/>
       <c r="L268" s="7"/>
     </row>
@@ -11949,7 +12552,9 @@
         <v>924</v>
       </c>
       <c r="I269" s="4"/>
-      <c r="J269" s="6"/>
+      <c r="J269" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K269" s="7"/>
       <c r="L269" s="7"/>
     </row>
@@ -11973,7 +12578,9 @@
       <c r="G270" s="3"/>
       <c r="H270" s="4"/>
       <c r="I270" s="4"/>
-      <c r="J270" s="6"/>
+      <c r="J270" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K270" s="7"/>
       <c r="L270" s="7"/>
     </row>
@@ -12003,7 +12610,9 @@
         <v>932</v>
       </c>
       <c r="I271" s="4"/>
-      <c r="J271" s="6"/>
+      <c r="J271" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K271" s="7"/>
       <c r="L271" s="7"/>
     </row>
@@ -12027,7 +12636,9 @@
       <c r="G272" s="3"/>
       <c r="H272" s="4"/>
       <c r="I272" s="4"/>
-      <c r="J272" s="6"/>
+      <c r="J272" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K272" s="7"/>
       <c r="L272" s="7"/>
     </row>
@@ -12057,7 +12668,9 @@
         <v>940</v>
       </c>
       <c r="I273" s="4"/>
-      <c r="J273" s="6"/>
+      <c r="J273" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K273" s="7"/>
       <c r="L273" s="7"/>
     </row>
@@ -12083,7 +12696,9 @@
       <c r="G274" s="3"/>
       <c r="H274" s="4"/>
       <c r="I274" s="4"/>
-      <c r="J274" s="6"/>
+      <c r="J274" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K274" s="7"/>
       <c r="L274" s="7"/>
     </row>
@@ -12113,7 +12728,9 @@
         <v>948</v>
       </c>
       <c r="I275" s="4"/>
-      <c r="J275" s="6"/>
+      <c r="J275" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K275" s="7"/>
       <c r="L275" s="7"/>
     </row>
@@ -12137,7 +12754,9 @@
       <c r="G276" s="3"/>
       <c r="H276" s="4"/>
       <c r="I276" s="4"/>
-      <c r="J276" s="6"/>
+      <c r="J276" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K276" s="7"/>
       <c r="L276" s="7"/>
     </row>
@@ -12167,7 +12786,9 @@
         <v>956</v>
       </c>
       <c r="I277" s="4"/>
-      <c r="J277" s="6"/>
+      <c r="J277" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K277" s="7"/>
       <c r="L277" s="7"/>
     </row>
@@ -12191,7 +12812,9 @@
       <c r="G278" s="3"/>
       <c r="H278" s="4"/>
       <c r="I278" s="4"/>
-      <c r="J278" s="6"/>
+      <c r="J278" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K278" s="7"/>
       <c r="L278" s="7"/>
     </row>
@@ -12221,7 +12844,9 @@
         <v>964</v>
       </c>
       <c r="I279" s="4"/>
-      <c r="J279" s="6"/>
+      <c r="J279" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K279" s="7"/>
       <c r="L279" s="7"/>
     </row>
@@ -12245,7 +12870,9 @@
       <c r="G280" s="3"/>
       <c r="H280" s="4"/>
       <c r="I280" s="4"/>
-      <c r="J280" s="6"/>
+      <c r="J280" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K280" s="7"/>
       <c r="L280" s="7"/>
     </row>
@@ -12275,7 +12902,9 @@
         <v>972</v>
       </c>
       <c r="I281" s="4"/>
-      <c r="J281" s="6"/>
+      <c r="J281" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K281" s="7"/>
       <c r="L281" s="7"/>
     </row>
@@ -12299,7 +12928,9 @@
       <c r="G282" s="3"/>
       <c r="H282" s="4"/>
       <c r="I282" s="4"/>
-      <c r="J282" s="6"/>
+      <c r="J282" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K282" s="7"/>
       <c r="L282" s="7"/>
     </row>
@@ -12329,7 +12960,9 @@
         <v>979</v>
       </c>
       <c r="I283" s="4"/>
-      <c r="J283" s="6"/>
+      <c r="J283" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K283" s="7"/>
       <c r="L283" s="7"/>
     </row>
@@ -12355,7 +12988,9 @@
       <c r="G284" s="3"/>
       <c r="H284" s="4"/>
       <c r="I284" s="4"/>
-      <c r="J284" s="6"/>
+      <c r="J284" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K284" s="7"/>
       <c r="L284" s="7"/>
     </row>
@@ -12385,7 +13020,9 @@
         <v>987</v>
       </c>
       <c r="I285" s="4"/>
-      <c r="J285" s="6"/>
+      <c r="J285" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K285" s="7"/>
       <c r="L285" s="7"/>
     </row>
@@ -12413,7 +13050,9 @@
       <c r="I286" s="10" t="s">
         <v>991</v>
       </c>
-      <c r="J286" s="6"/>
+      <c r="J286" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K286" s="7"/>
       <c r="L286" s="7"/>
     </row>
@@ -12443,7 +13082,9 @@
         <v>996</v>
       </c>
       <c r="I287" s="4"/>
-      <c r="J287" s="6"/>
+      <c r="J287" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K287" s="7"/>
       <c r="L287" s="7"/>
     </row>
@@ -12473,7 +13114,9 @@
         <v>470</v>
       </c>
       <c r="I288" s="4"/>
-      <c r="J288" s="6"/>
+      <c r="J288" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K288" s="7"/>
       <c r="L288" s="7"/>
     </row>
@@ -12503,7 +13146,9 @@
         <v>1005</v>
       </c>
       <c r="I289" s="4"/>
-      <c r="J289" s="6"/>
+      <c r="J289" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K289" s="7"/>
       <c r="L289" s="7"/>
     </row>
@@ -12531,7 +13176,9 @@
         <v>1009</v>
       </c>
       <c r="I290" s="4"/>
-      <c r="J290" s="6"/>
+      <c r="J290" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K290" s="7"/>
       <c r="L290" s="7"/>
     </row>
@@ -12561,7 +13208,9 @@
         <v>1014</v>
       </c>
       <c r="I291" s="4"/>
-      <c r="J291" s="6"/>
+      <c r="J291" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K291" s="7"/>
       <c r="L291" s="7"/>
     </row>
@@ -12591,7 +13240,9 @@
         <v>470</v>
       </c>
       <c r="I292" s="4"/>
-      <c r="J292" s="6"/>
+      <c r="J292" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K292" s="7"/>
       <c r="L292" s="7"/>
     </row>
@@ -12621,7 +13272,9 @@
         <v>1023</v>
       </c>
       <c r="I293" s="4"/>
-      <c r="J293" s="6"/>
+      <c r="J293" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K293" s="7"/>
       <c r="L293" s="7"/>
     </row>
@@ -12645,7 +13298,9 @@
       <c r="G294" s="3"/>
       <c r="H294" s="4"/>
       <c r="I294" s="4"/>
-      <c r="J294" s="6"/>
+      <c r="J294" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K294" s="7"/>
       <c r="L294" s="7"/>
     </row>
@@ -12675,7 +13330,9 @@
         <v>1030</v>
       </c>
       <c r="I295" s="4"/>
-      <c r="J295" s="6"/>
+      <c r="J295" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K295" s="7"/>
       <c r="L295" s="7"/>
     </row>
@@ -12701,7 +13358,9 @@
       <c r="G296" s="3"/>
       <c r="H296" s="4"/>
       <c r="I296" s="4"/>
-      <c r="J296" s="6"/>
+      <c r="J296" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K296" s="7"/>
       <c r="L296" s="7"/>
     </row>
@@ -12731,7 +13390,9 @@
         <v>1038</v>
       </c>
       <c r="I297" s="4"/>
-      <c r="J297" s="6"/>
+      <c r="J297" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K297" s="7"/>
       <c r="L297" s="7"/>
     </row>
@@ -12757,7 +13418,9 @@
       <c r="G298" s="3"/>
       <c r="H298" s="4"/>
       <c r="I298" s="4"/>
-      <c r="J298" s="6"/>
+      <c r="J298" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K298" s="7"/>
       <c r="L298" s="7"/>
     </row>
@@ -12787,7 +13450,9 @@
         <v>1046</v>
       </c>
       <c r="I299" s="4"/>
-      <c r="J299" s="6"/>
+      <c r="J299" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K299" s="7"/>
       <c r="L299" s="7"/>
     </row>
@@ -12811,7 +13476,9 @@
       <c r="G300" s="3"/>
       <c r="H300" s="4"/>
       <c r="I300" s="4"/>
-      <c r="J300" s="6"/>
+      <c r="J300" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K300" s="7"/>
       <c r="L300" s="7"/>
     </row>
@@ -12841,7 +13508,9 @@
         <v>1054</v>
       </c>
       <c r="I301" s="4"/>
-      <c r="J301" s="6"/>
+      <c r="J301" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K301" s="7"/>
       <c r="L301" s="7"/>
     </row>
@@ -12871,7 +13540,9 @@
         <v>470</v>
       </c>
       <c r="I302" s="4"/>
-      <c r="J302" s="6"/>
+      <c r="J302" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K302" s="7"/>
       <c r="L302" s="7"/>
     </row>
@@ -12901,7 +13572,9 @@
         <v>758</v>
       </c>
       <c r="I303" s="4"/>
-      <c r="J303" s="6"/>
+      <c r="J303" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K303" s="7"/>
       <c r="L303" s="7"/>
     </row>
@@ -12925,7 +13598,9 @@
       <c r="G304" s="3"/>
       <c r="H304" s="4"/>
       <c r="I304" s="4"/>
-      <c r="J304" s="6"/>
+      <c r="J304" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K304" s="7"/>
       <c r="L304" s="7"/>
     </row>
@@ -12955,7 +13630,9 @@
         <v>1069</v>
       </c>
       <c r="I305" s="4"/>
-      <c r="J305" s="6"/>
+      <c r="J305" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K305" s="7"/>
       <c r="L305" s="7"/>
     </row>
@@ -12979,7 +13656,9 @@
       <c r="G306" s="3"/>
       <c r="H306" s="4"/>
       <c r="I306" s="4"/>
-      <c r="J306" s="6"/>
+      <c r="J306" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K306" s="7"/>
       <c r="L306" s="7"/>
     </row>
@@ -13009,7 +13688,9 @@
         <v>1005</v>
       </c>
       <c r="I307" s="4"/>
-      <c r="J307" s="6"/>
+      <c r="J307" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K307" s="7"/>
       <c r="L307" s="7"/>
     </row>
@@ -13033,7 +13714,9 @@
       <c r="G308" s="3"/>
       <c r="H308" s="4"/>
       <c r="I308" s="4"/>
-      <c r="J308" s="6"/>
+      <c r="J308" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K308" s="7"/>
       <c r="L308" s="7"/>
     </row>
@@ -13063,7 +13746,9 @@
         <v>1084</v>
       </c>
       <c r="I309" s="4"/>
-      <c r="J309" s="6"/>
+      <c r="J309" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K309" s="7"/>
       <c r="L309" s="7"/>
     </row>
@@ -13093,7 +13778,9 @@
         <v>470</v>
       </c>
       <c r="I310" s="4"/>
-      <c r="J310" s="6"/>
+      <c r="J310" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K310" s="7"/>
       <c r="L310" s="7"/>
     </row>
@@ -13123,7 +13810,9 @@
         <v>1093</v>
       </c>
       <c r="I311" s="4"/>
-      <c r="J311" s="6"/>
+      <c r="J311" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K311" s="7"/>
       <c r="L311" s="7"/>
     </row>
@@ -13147,7 +13836,9 @@
       <c r="G312" s="3"/>
       <c r="H312" s="4"/>
       <c r="I312" s="4"/>
-      <c r="J312" s="6"/>
+      <c r="J312" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K312" s="7"/>
       <c r="L312" s="7"/>
     </row>
@@ -13177,7 +13868,9 @@
         <v>1101</v>
       </c>
       <c r="I313" s="4"/>
-      <c r="J313" s="6"/>
+      <c r="J313" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K313" s="7"/>
       <c r="L313" s="7"/>
     </row>
@@ -13203,7 +13896,9 @@
       <c r="G314" s="3"/>
       <c r="H314" s="4"/>
       <c r="I314" s="4"/>
-      <c r="J314" s="6"/>
+      <c r="J314" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K314" s="7"/>
       <c r="L314" s="7"/>
     </row>
@@ -13233,7 +13928,9 @@
         <v>1109</v>
       </c>
       <c r="I315" s="4"/>
-      <c r="J315" s="6"/>
+      <c r="J315" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K315" s="7"/>
       <c r="L315" s="7"/>
     </row>
@@ -13257,7 +13954,9 @@
       <c r="G316" s="3"/>
       <c r="H316" s="4"/>
       <c r="I316" s="4"/>
-      <c r="J316" s="6"/>
+      <c r="J316" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K316" s="7"/>
       <c r="L316" s="7"/>
     </row>
@@ -13287,7 +13986,9 @@
         <v>1116</v>
       </c>
       <c r="I317" s="4"/>
-      <c r="J317" s="6"/>
+      <c r="J317" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K317" s="7"/>
       <c r="L317" s="7"/>
     </row>
@@ -13313,7 +14014,9 @@
       <c r="G318" s="3"/>
       <c r="H318" s="4"/>
       <c r="I318" s="4"/>
-      <c r="J318" s="6"/>
+      <c r="J318" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K318" s="7"/>
       <c r="L318" s="7"/>
     </row>
@@ -13343,7 +14046,9 @@
         <v>1124</v>
       </c>
       <c r="I319" s="4"/>
-      <c r="J319" s="6"/>
+      <c r="J319" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K319" s="7"/>
       <c r="L319" s="7"/>
     </row>
@@ -13369,7 +14074,9 @@
       <c r="G320" s="3"/>
       <c r="H320" s="4"/>
       <c r="I320" s="4"/>
-      <c r="J320" s="6"/>
+      <c r="J320" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K320" s="7"/>
       <c r="L320" s="7"/>
     </row>
@@ -13399,7 +14106,9 @@
         <v>870</v>
       </c>
       <c r="I321" s="4"/>
-      <c r="J321" s="6"/>
+      <c r="J321" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K321" s="7"/>
       <c r="L321" s="7"/>
     </row>
@@ -13429,7 +14138,9 @@
         <v>1136</v>
       </c>
       <c r="I322" s="4"/>
-      <c r="J322" s="6"/>
+      <c r="J322" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K322" s="7"/>
       <c r="L322" s="7"/>
     </row>
@@ -13459,7 +14170,9 @@
         <v>1141</v>
       </c>
       <c r="I323" s="4"/>
-      <c r="J323" s="6"/>
+      <c r="J323" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K323" s="7"/>
       <c r="L323" s="7"/>
     </row>
@@ -13485,7 +14198,9 @@
       <c r="G324" s="3"/>
       <c r="H324" s="4"/>
       <c r="I324" s="4"/>
-      <c r="J324" s="6"/>
+      <c r="J324" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K324" s="7"/>
       <c r="L324" s="7"/>
     </row>
@@ -13515,7 +14230,9 @@
         <v>1149</v>
       </c>
       <c r="I325" s="4"/>
-      <c r="J325" s="6"/>
+      <c r="J325" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K325" s="7"/>
       <c r="L325" s="7"/>
     </row>
@@ -13545,7 +14262,9 @@
         <v>470</v>
       </c>
       <c r="I326" s="4"/>
-      <c r="J326" s="6"/>
+      <c r="J326" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K326" s="7"/>
       <c r="L326" s="7"/>
     </row>
@@ -13575,7 +14294,9 @@
         <v>1158</v>
       </c>
       <c r="I327" s="4"/>
-      <c r="J327" s="6"/>
+      <c r="J327" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K327" s="7"/>
       <c r="L327" s="7"/>
     </row>
@@ -13605,7 +14326,9 @@
         <v>470</v>
       </c>
       <c r="I328" s="4"/>
-      <c r="J328" s="6"/>
+      <c r="J328" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K328" s="7"/>
       <c r="L328" s="7"/>
     </row>
@@ -13635,7 +14358,9 @@
         <v>1054</v>
       </c>
       <c r="I329" s="4"/>
-      <c r="J329" s="6"/>
+      <c r="J329" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K329" s="7"/>
       <c r="L329" s="7"/>
     </row>
@@ -13661,7 +14386,9 @@
       <c r="G330" s="3"/>
       <c r="H330" s="4"/>
       <c r="I330" s="4"/>
-      <c r="J330" s="6"/>
+      <c r="J330" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K330" s="7"/>
       <c r="L330" s="7"/>
     </row>
@@ -13691,7 +14418,9 @@
         <v>862</v>
       </c>
       <c r="I331" s="4"/>
-      <c r="J331" s="6"/>
+      <c r="J331" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K331" s="7"/>
       <c r="L331" s="7"/>
     </row>
@@ -13715,7 +14444,9 @@
       <c r="G332" s="3"/>
       <c r="H332" s="4"/>
       <c r="I332" s="4"/>
-      <c r="J332" s="6"/>
+      <c r="J332" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K332" s="7"/>
       <c r="L332" s="7"/>
     </row>
@@ -13745,7 +14476,9 @@
         <v>1179</v>
       </c>
       <c r="I333" s="4"/>
-      <c r="J333" s="6"/>
+      <c r="J333" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K333" s="7"/>
       <c r="L333" s="7"/>
     </row>
@@ -13771,7 +14504,9 @@
       <c r="G334" s="3"/>
       <c r="H334" s="4"/>
       <c r="I334" s="4"/>
-      <c r="J334" s="6"/>
+      <c r="J334" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K334" s="7"/>
       <c r="L334" s="7"/>
     </row>
@@ -13801,7 +14536,9 @@
         <v>1187</v>
       </c>
       <c r="I335" s="4"/>
-      <c r="J335" s="6"/>
+      <c r="J335" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K335" s="7"/>
       <c r="L335" s="7"/>
     </row>
@@ -13831,7 +14568,9 @@
         <v>1192</v>
       </c>
       <c r="I336" s="4"/>
-      <c r="J336" s="6"/>
+      <c r="J336" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K336" s="7"/>
       <c r="L336" s="7"/>
     </row>
@@ -13863,7 +14602,9 @@
       <c r="I337" s="10" t="s">
         <v>880</v>
       </c>
-      <c r="J337" s="6"/>
+      <c r="J337" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K337" s="7"/>
       <c r="L337" s="7"/>
     </row>
@@ -13891,7 +14632,9 @@
       <c r="I338" s="10" t="s">
         <v>1202</v>
       </c>
-      <c r="J338" s="6"/>
+      <c r="J338" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K338" s="7"/>
       <c r="L338" s="7"/>
     </row>
@@ -13921,7 +14664,9 @@
         <v>1054</v>
       </c>
       <c r="I339" s="4"/>
-      <c r="J339" s="6"/>
+      <c r="J339" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K339" s="7"/>
       <c r="L339" s="7"/>
     </row>
@@ -13949,7 +14694,9 @@
       <c r="I340" s="10" t="s">
         <v>1210</v>
       </c>
-      <c r="J340" s="6"/>
+      <c r="J340" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K340" s="7"/>
       <c r="L340" s="7"/>
     </row>
@@ -13979,7 +14726,9 @@
         <v>1215</v>
       </c>
       <c r="I341" s="4"/>
-      <c r="J341" s="6"/>
+      <c r="J341" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K341" s="7"/>
       <c r="L341" s="7"/>
     </row>
@@ -14003,7 +14752,9 @@
       <c r="G342" s="3"/>
       <c r="H342" s="4"/>
       <c r="I342" s="4"/>
-      <c r="J342" s="6"/>
+      <c r="J342" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K342" s="7"/>
       <c r="L342" s="7"/>
     </row>
@@ -14033,7 +14784,9 @@
         <v>1223</v>
       </c>
       <c r="I343" s="4"/>
-      <c r="J343" s="6"/>
+      <c r="J343" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K343" s="7"/>
       <c r="L343" s="7"/>
     </row>
@@ -14057,7 +14810,9 @@
       <c r="G344" s="3"/>
       <c r="H344" s="4"/>
       <c r="I344" s="4"/>
-      <c r="J344" s="6"/>
+      <c r="J344" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K344" s="7"/>
       <c r="L344" s="7"/>
     </row>
@@ -14087,7 +14842,9 @@
         <v>1231</v>
       </c>
       <c r="I345" s="4"/>
-      <c r="J345" s="6"/>
+      <c r="J345" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K345" s="7"/>
       <c r="L345" s="7"/>
     </row>
@@ -14117,7 +14874,9 @@
         <v>1236</v>
       </c>
       <c r="I346" s="4"/>
-      <c r="J346" s="6"/>
+      <c r="J346" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K346" s="7"/>
       <c r="L346" s="7"/>
     </row>
@@ -14147,7 +14906,9 @@
         <v>1241</v>
       </c>
       <c r="I347" s="4"/>
-      <c r="J347" s="6"/>
+      <c r="J347" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K347" s="7"/>
       <c r="L347" s="7"/>
     </row>
@@ -14177,7 +14938,9 @@
         <v>1246</v>
       </c>
       <c r="I348" s="4"/>
-      <c r="J348" s="6"/>
+      <c r="J348" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K348" s="7"/>
       <c r="L348" s="7"/>
     </row>
@@ -14207,7 +14970,9 @@
         <v>1251</v>
       </c>
       <c r="I349" s="4"/>
-      <c r="J349" s="6"/>
+      <c r="J349" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K349" s="7"/>
       <c r="L349" s="7"/>
     </row>
@@ -14239,9 +15004,15 @@
       <c r="I350" s="10" t="s">
         <v>1257</v>
       </c>
-      <c r="J350" s="6"/>
-      <c r="K350" s="7"/>
-      <c r="L350" s="7"/>
+      <c r="J350" s="6" t="s">
+        <v>1463</v>
+      </c>
+      <c r="K350" s="7" t="s">
+        <v>1476</v>
+      </c>
+      <c r="L350" s="7" t="s">
+        <v>1054</v>
+      </c>
     </row>
     <row r="351" spans="1:12" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A351" s="3" t="s">
@@ -14269,7 +15040,9 @@
         <v>1005</v>
       </c>
       <c r="I351" s="4"/>
-      <c r="J351" s="6"/>
+      <c r="J351" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K351" s="7"/>
       <c r="L351" s="7"/>
     </row>
@@ -14299,7 +15072,9 @@
         <v>1266</v>
       </c>
       <c r="I352" s="4"/>
-      <c r="J352" s="6"/>
+      <c r="J352" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K352" s="7"/>
       <c r="L352" s="7"/>
     </row>
@@ -14329,7 +15104,9 @@
         <v>1271</v>
       </c>
       <c r="I353" s="4"/>
-      <c r="J353" s="6"/>
+      <c r="J353" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K353" s="7"/>
       <c r="L353" s="7"/>
     </row>
@@ -14359,7 +15136,9 @@
         <v>1276</v>
       </c>
       <c r="I354" s="4"/>
-      <c r="J354" s="6"/>
+      <c r="J354" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K354" s="7"/>
       <c r="L354" s="7"/>
     </row>
@@ -14385,7 +15164,9 @@
       <c r="G355" s="3"/>
       <c r="H355" s="4"/>
       <c r="I355" s="4"/>
-      <c r="J355" s="6"/>
+      <c r="J355" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K355" s="7"/>
       <c r="L355" s="7"/>
     </row>
@@ -14411,7 +15192,9 @@
       <c r="G356" s="3"/>
       <c r="H356" s="4"/>
       <c r="I356" s="4"/>
-      <c r="J356" s="6"/>
+      <c r="J356" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K356" s="7"/>
       <c r="L356" s="7"/>
     </row>
@@ -14437,7 +15220,9 @@
       <c r="G357" s="3"/>
       <c r="H357" s="4"/>
       <c r="I357" s="4"/>
-      <c r="J357" s="6"/>
+      <c r="J357" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K357" s="7"/>
       <c r="L357" s="7"/>
     </row>
@@ -14467,7 +15252,9 @@
         <v>1290</v>
       </c>
       <c r="I358" s="4"/>
-      <c r="J358" s="6"/>
+      <c r="J358" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K358" s="7"/>
       <c r="L358" s="7"/>
     </row>
@@ -14493,7 +15280,9 @@
       <c r="G359" s="3"/>
       <c r="H359" s="4"/>
       <c r="I359" s="4"/>
-      <c r="J359" s="6"/>
+      <c r="J359" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K359" s="7"/>
       <c r="L359" s="7"/>
     </row>
@@ -14519,7 +15308,9 @@
       <c r="G360" s="3"/>
       <c r="H360" s="4"/>
       <c r="I360" s="4"/>
-      <c r="J360" s="6"/>
+      <c r="J360" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K360" s="7"/>
       <c r="L360" s="7"/>
     </row>
@@ -14545,7 +15336,9 @@
       <c r="G361" s="3"/>
       <c r="H361" s="4"/>
       <c r="I361" s="4"/>
-      <c r="J361" s="6"/>
+      <c r="J361" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K361" s="7"/>
       <c r="L361" s="7"/>
     </row>
@@ -14571,7 +15364,9 @@
       <c r="G362" s="3"/>
       <c r="H362" s="4"/>
       <c r="I362" s="4"/>
-      <c r="J362" s="6"/>
+      <c r="J362" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K362" s="7"/>
       <c r="L362" s="7"/>
     </row>
@@ -14601,7 +15396,9 @@
         <v>1307</v>
       </c>
       <c r="I363" s="4"/>
-      <c r="J363" s="6"/>
+      <c r="J363" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K363" s="7"/>
       <c r="L363" s="7"/>
     </row>
@@ -14631,7 +15428,9 @@
         <v>1312</v>
       </c>
       <c r="I364" s="4"/>
-      <c r="J364" s="6"/>
+      <c r="J364" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K364" s="7"/>
       <c r="L364" s="7"/>
     </row>
@@ -14661,7 +15460,9 @@
         <v>1317</v>
       </c>
       <c r="I365" s="4"/>
-      <c r="J365" s="6"/>
+      <c r="J365" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K365" s="7"/>
       <c r="L365" s="7"/>
     </row>
@@ -14691,7 +15492,9 @@
         <v>1322</v>
       </c>
       <c r="I366" s="4"/>
-      <c r="J366" s="6"/>
+      <c r="J366" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K366" s="7"/>
       <c r="L366" s="7"/>
     </row>
@@ -14721,7 +15524,9 @@
         <v>1327</v>
       </c>
       <c r="I367" s="4"/>
-      <c r="J367" s="6"/>
+      <c r="J367" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K367" s="7"/>
       <c r="L367" s="7"/>
     </row>
@@ -14751,7 +15556,9 @@
         <v>1332</v>
       </c>
       <c r="I368" s="4"/>
-      <c r="J368" s="6"/>
+      <c r="J368" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K368" s="7"/>
       <c r="L368" s="7"/>
     </row>
@@ -14781,7 +15588,9 @@
         <v>704</v>
       </c>
       <c r="I369" s="4"/>
-      <c r="J369" s="6"/>
+      <c r="J369" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K369" s="7"/>
       <c r="L369" s="7"/>
     </row>
@@ -14811,7 +15620,9 @@
         <v>1341</v>
       </c>
       <c r="I370" s="4"/>
-      <c r="J370" s="6"/>
+      <c r="J370" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K370" s="7"/>
       <c r="L370" s="7"/>
     </row>
@@ -14841,7 +15652,9 @@
         <v>1005</v>
       </c>
       <c r="I371" s="4"/>
-      <c r="J371" s="6"/>
+      <c r="J371" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K371" s="7"/>
       <c r="L371" s="7"/>
     </row>
@@ -14871,7 +15684,9 @@
         <v>1350</v>
       </c>
       <c r="I372" s="4"/>
-      <c r="J372" s="6"/>
+      <c r="J372" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K372" s="7"/>
       <c r="L372" s="7"/>
     </row>
@@ -14901,7 +15716,9 @@
         <v>1005</v>
       </c>
       <c r="I373" s="4"/>
-      <c r="J373" s="6"/>
+      <c r="J373" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K373" s="7"/>
       <c r="L373" s="7"/>
     </row>
@@ -14931,7 +15748,9 @@
         <v>1359</v>
       </c>
       <c r="I374" s="4"/>
-      <c r="J374" s="6"/>
+      <c r="J374" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K374" s="7"/>
       <c r="L374" s="7"/>
     </row>
@@ -14961,7 +15780,9 @@
         <v>1364</v>
       </c>
       <c r="I375" s="4"/>
-      <c r="J375" s="6"/>
+      <c r="J375" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K375" s="7"/>
       <c r="L375" s="7"/>
     </row>
@@ -14993,7 +15814,9 @@
       <c r="I376" s="10" t="s">
         <v>1369</v>
       </c>
-      <c r="J376" s="6"/>
+      <c r="J376" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K376" s="7"/>
       <c r="L376" s="7"/>
     </row>
@@ -15023,7 +15846,9 @@
         <v>1374</v>
       </c>
       <c r="I377" s="4"/>
-      <c r="J377" s="6"/>
+      <c r="J377" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K377" s="7"/>
       <c r="L377" s="7"/>
     </row>
@@ -15053,7 +15878,9 @@
         <v>862</v>
       </c>
       <c r="I378" s="4"/>
-      <c r="J378" s="6"/>
+      <c r="J378" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K378" s="7"/>
       <c r="L378" s="7"/>
     </row>
@@ -15083,7 +15910,9 @@
         <v>1383</v>
       </c>
       <c r="I379" s="4"/>
-      <c r="J379" s="6"/>
+      <c r="J379" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K379" s="7"/>
       <c r="L379" s="7"/>
     </row>
@@ -15113,7 +15942,9 @@
         <v>1388</v>
       </c>
       <c r="I380" s="4"/>
-      <c r="J380" s="6"/>
+      <c r="J380" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K380" s="7"/>
       <c r="L380" s="7"/>
     </row>
@@ -15143,7 +15974,9 @@
         <v>1393</v>
       </c>
       <c r="I381" s="4"/>
-      <c r="J381" s="6"/>
+      <c r="J381" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K381" s="7"/>
       <c r="L381" s="7"/>
     </row>
@@ -15173,7 +16006,9 @@
         <v>1398</v>
       </c>
       <c r="I382" s="4"/>
-      <c r="J382" s="6"/>
+      <c r="J382" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K382" s="7"/>
       <c r="L382" s="7"/>
     </row>
@@ -15203,7 +16038,9 @@
         <v>1403</v>
       </c>
       <c r="I383" s="4"/>
-      <c r="J383" s="6"/>
+      <c r="J383" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K383" s="7"/>
       <c r="L383" s="7"/>
     </row>
@@ -15233,7 +16070,9 @@
         <v>1408</v>
       </c>
       <c r="I384" s="4"/>
-      <c r="J384" s="6"/>
+      <c r="J384" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K384" s="7"/>
       <c r="L384" s="7"/>
     </row>
@@ -15263,7 +16102,9 @@
         <v>1005</v>
       </c>
       <c r="I385" s="4"/>
-      <c r="J385" s="6"/>
+      <c r="J385" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K385" s="7"/>
       <c r="L385" s="7"/>
     </row>
@@ -15293,7 +16134,9 @@
         <v>1417</v>
       </c>
       <c r="I386" s="4"/>
-      <c r="J386" s="6"/>
+      <c r="J386" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K386" s="7"/>
       <c r="L386" s="7"/>
     </row>
@@ -15323,7 +16166,9 @@
         <v>1422</v>
       </c>
       <c r="I387" s="4"/>
-      <c r="J387" s="6"/>
+      <c r="J387" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K387" s="7"/>
       <c r="L387" s="7"/>
     </row>
@@ -15353,7 +16198,9 @@
         <v>1427</v>
       </c>
       <c r="I388" s="4"/>
-      <c r="J388" s="6"/>
+      <c r="J388" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K388" s="7"/>
       <c r="L388" s="7"/>
     </row>
@@ -15383,7 +16230,9 @@
         <v>1432</v>
       </c>
       <c r="I389" s="4"/>
-      <c r="J389" s="6"/>
+      <c r="J389" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K389" s="7"/>
       <c r="L389" s="7"/>
     </row>
@@ -15413,7 +16262,9 @@
         <v>1437</v>
       </c>
       <c r="I390" s="4"/>
-      <c r="J390" s="6"/>
+      <c r="J390" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K390" s="7"/>
       <c r="L390" s="7"/>
     </row>
@@ -15443,7 +16294,9 @@
         <v>1442</v>
       </c>
       <c r="I391" s="4"/>
-      <c r="J391" s="6"/>
+      <c r="J391" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K391" s="7"/>
       <c r="L391" s="7"/>
     </row>
@@ -15475,7 +16328,9 @@
       <c r="I392" s="10" t="s">
         <v>1448</v>
       </c>
-      <c r="J392" s="6"/>
+      <c r="J392" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="K392" s="7"/>
       <c r="L392" s="7"/>
     </row>

</xml_diff>